<commit_message>
Update plan-site to room-based pricing model (base package + room builder, tiers as example starting points); align pricing workbook with PRD 1 expansion rule
</commit_message>
<xml_diff>
--- a/pricing/OneHome_pricing_model.xlsx
+++ b/pricing/OneHome_pricing_model.xlsx
@@ -45,19 +45,19 @@
     <t xml:space="preserve">תעריף שעת עבודה של גיא (₪)</t>
   </si>
   <si>
-    <t xml:space="preserve">הערכה. תעריף טכנאי/אינטגרטור בישראל; לכייל מול זמנים בפועל אצל 3 הלקוחות הראשונים.</t>
+    <t xml:space="preserve">מתוך PRD 1 (מדיניות הרחבות, נסגר): 180 ₪ לשעה.</t>
   </si>
   <si>
     <t xml:space="preserve">מרווח על חומרה (%)</t>
   </si>
   <si>
-    <t xml:space="preserve">כיסוי רכש, משלוח, החלפות באחריות והון חוזר. לא רווח נטו.</t>
+    <t xml:space="preserve">מתוך PRD 1 (מדיניות הרחבות, נסגר): עלות חומרה ×1.3.</t>
   </si>
   <si>
     <t xml:space="preserve">דמי ביקור חשמלאי (₪, פעם אחת להתקנה)</t>
   </si>
   <si>
-    <t xml:space="preserve">הערכה. חל רק אם יש לפחות פריט אחד שדורש חשמלאי (PRD 1 סעיף F).</t>
+    <t xml:space="preserve">מתוך PRD 1 (מדיניות הרחבות, נסגר): +495 ₪ אם נדרש חשמלאי. בהתקנה מלאה נוספת גם עבודת חשמלאי לכל נקודה (עמודה F בקטלוג) — הערכה, לאמת מול החשמלאי.</t>
   </si>
   <si>
     <t xml:space="preserve">שעות עבודה בחבילה הבסיסית</t>
@@ -636,20 +636,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -657,95 +661,95 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1004,144 +1008,144 @@
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="95"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="6" t="n">
-        <v>250</v>
-      </c>
-      <c r="C5" s="5" t="s">
+      <c r="B5" s="7" t="n">
+        <v>180</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="7" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C6" s="5" t="s">
+      <c r="B6" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="7" t="n">
+        <v>495</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="9" t="n">
         <v>3.7</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1162,869 +1166,869 @@
   <dimension ref="A1:J28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="55"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="12" t="n">
         <v>900</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="13" t="n">
+      <c r="H5" s="14" t="n">
         <f aca="false">ROUNDUP((D5*(1+הנחות!$B$6)+E5/60*הנחות!$B$5+F5)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>1080</v>
-      </c>
-      <c r="I5" s="10" t="s">
+        <v>1170</v>
+      </c>
+      <c r="I5" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="J5" s="10" t="s">
+      <c r="J5" s="11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="12" t="n">
         <v>250</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="13" t="n">
+      <c r="H6" s="14" t="n">
         <f aca="false">ROUNDUP((D6*(1+הנחות!$B$6)+E6/60*הנחות!$B$5+F6)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>300</v>
-      </c>
-      <c r="I6" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I6" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="J6" s="11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="F7" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="13" t="n">
+      <c r="G7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="14" t="n">
         <f aca="false">ROUNDUP((D7*(1+הנחות!$B$6)+E7/60*הנחות!$B$5+F7)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>610</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="J7" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="12" t="n">
         <v>130</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="13" t="n">
+      <c r="G8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="14" t="n">
         <f aca="false">ROUNDUP((D8*(1+הנחות!$B$6)+E8/60*הנחות!$B$5+F8)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>200</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J8" s="10"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="J8" s="11"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="12" t="n">
         <v>110</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="F9" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="13" t="n">
+      <c r="G9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="14" t="n">
         <f aca="false">ROUNDUP((D9*(1+הנחות!$B$6)+E9/60*הנחות!$B$5+F9)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>260</v>
-      </c>
-      <c r="I9" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="I9" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="11" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="12" t="n">
         <v>90</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="13" t="n">
+      <c r="G10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="14" t="n">
         <f aca="false">ROUNDUP((D10*(1+הנחות!$B$6)+E10/60*הנחות!$B$5+F10)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>150</v>
       </c>
-      <c r="I10" s="10" t="s">
+      <c r="I10" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="10"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="J10" s="11"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="12" t="n">
         <v>200</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="F11" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="13" t="n">
+      <c r="G11" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="14" t="n">
         <f aca="false">ROUNDUP((D11*(1+הנחות!$B$6)+E11/60*הנחות!$B$5+F11)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>310</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="I11" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J11" s="10"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
+      <c r="J11" s="11"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="12" t="n">
         <v>90</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="13" t="n">
+      <c r="G12" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="14" t="n">
         <f aca="false">ROUNDUP((D12*(1+הנחות!$B$6)+E12/60*הנחות!$B$5+F12)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>150</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J12" s="10" t="s">
+      <c r="J12" s="11" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="12" t="n">
         <v>200</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="F13" s="11" t="n">
+      <c r="F13" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="13" t="n">
+      <c r="G13" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="14" t="n">
         <f aca="false">ROUNDUP((D13*(1+הנחות!$B$6)+E13/60*הנחות!$B$5+F13)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>310</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="I13" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J13" s="10" t="s">
+      <c r="J13" s="11" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="12" t="n">
         <v>350</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="13" t="n">
         <v>20</v>
       </c>
-      <c r="F14" s="11" t="n">
+      <c r="F14" s="12" t="n">
         <v>300</v>
       </c>
-      <c r="G14" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H14" s="13" t="n">
+      <c r="G14" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="14" t="n">
         <f aca="false">ROUNDUP((D14*(1+הנחות!$B$6)+E14/60*הנחות!$B$5+F14)/הנחות!$B$10,0)*הנחות!$B$10</f>
+        <v>820</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="J14" s="11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>380</v>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>250</v>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="14" t="n">
+        <f aca="false">ROUNDUP((D15*(1+הנחות!$B$6)+E15/60*הנחות!$B$5+F15)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>810</v>
       </c>
-      <c r="I14" s="10" t="s">
+      <c r="I15" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="J14" s="10" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B15" s="10" t="s">
+      <c r="J15" s="11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="D15" s="11" t="n">
-        <v>380</v>
-      </c>
-      <c r="E15" s="12" t="n">
+      <c r="C16" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>250</v>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <f aca="false">ROUNDUP((D16*(1+הנחות!$B$6)+E16/60*הנחות!$B$5+F16)/הנחות!$B$10,0)*הנחות!$B$10</f>
+        <v>690</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="J16" s="11" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>650</v>
+      </c>
+      <c r="E17" s="13" t="n">
         <v>20</v>
       </c>
-      <c r="F15" s="11" t="n">
-        <v>250</v>
-      </c>
-      <c r="G15" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H15" s="13" t="n">
-        <f aca="false">ROUNDUP((D15*(1+הנחות!$B$6)+E15/60*הנחות!$B$5+F15)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>790</v>
-      </c>
-      <c r="I15" s="10" t="s">
+      <c r="F17" s="12" t="n">
+        <v>350</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="14" t="n">
+        <f aca="false">ROUNDUP((D17*(1+הנחות!$B$6)+E17/60*הנחות!$B$5+F17)/הנחות!$B$10,0)*הנחות!$B$10</f>
+        <v>1260</v>
+      </c>
+      <c r="I17" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="J15" s="10" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="D16" s="11" t="n">
-        <v>300</v>
-      </c>
-      <c r="E16" s="12" t="n">
-        <v>15</v>
-      </c>
-      <c r="F16" s="11" t="n">
-        <v>250</v>
-      </c>
-      <c r="G16" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" s="13" t="n">
-        <f aca="false">ROUNDUP((D16*(1+הנחות!$B$6)+E16/60*הנחות!$B$5+F16)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>680</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="J16" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="D17" s="11" t="n">
-        <v>650</v>
-      </c>
-      <c r="E17" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>350</v>
-      </c>
-      <c r="G17" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="13" t="n">
-        <f aca="false">ROUNDUP((D17*(1+הנחות!$B$6)+E17/60*הנחות!$B$5+F17)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>1220</v>
-      </c>
-      <c r="I17" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="J17" s="10" t="s">
+      <c r="J17" s="11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D18" s="12" t="n">
         <v>110</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F18" s="11" t="n">
+      <c r="F18" s="12" t="n">
         <v>150</v>
       </c>
-      <c r="G18" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" s="13" t="n">
+      <c r="G18" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="14" t="n">
         <f aca="false">ROUNDUP((D18*(1+הנחות!$B$6)+E18/60*הנחות!$B$5+F18)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>330</v>
       </c>
-      <c r="I18" s="10" t="s">
+      <c r="I18" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J18" s="10" t="s">
+      <c r="J18" s="11" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="D19" s="11" t="n">
+      <c r="D19" s="12" t="n">
         <v>160</v>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="F19" s="11" t="n">
+      <c r="F19" s="12" t="n">
         <v>150</v>
       </c>
-      <c r="G19" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="13" t="n">
+      <c r="G19" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="14" t="n">
         <f aca="false">ROUNDUP((D19*(1+הנחות!$B$6)+E19/60*הנחות!$B$5+F19)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>410</v>
       </c>
-      <c r="I19" s="10" t="s">
+      <c r="I19" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J19" s="10" t="s">
+      <c r="J19" s="11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="D20" s="11" t="n">
+      <c r="D20" s="12" t="n">
         <v>170</v>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E20" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F20" s="11" t="n">
+      <c r="F20" s="12" t="n">
         <v>150</v>
       </c>
-      <c r="G20" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="13" t="n">
+      <c r="G20" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="14" t="n">
         <f aca="false">ROUNDUP((D20*(1+הנחות!$B$6)+E20/60*הנחות!$B$5+F20)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>400</v>
-      </c>
-      <c r="I20" s="10" t="s">
+        <v>410</v>
+      </c>
+      <c r="I20" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J20" s="10" t="s">
+      <c r="J20" s="11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="D21" s="11" t="n">
+      <c r="D21" s="12" t="n">
         <v>75</v>
       </c>
-      <c r="E21" s="12" t="n">
+      <c r="E21" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F21" s="11" t="n">
+      <c r="F21" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" s="13" t="n">
+      <c r="G21" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="14" t="n">
         <f aca="false">ROUNDUP((D21*(1+הנחות!$B$6)+E21/60*הנחות!$B$5+F21)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>140</v>
-      </c>
-      <c r="I21" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="I21" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J21" s="10" t="s">
+      <c r="J21" s="11" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D22" s="11" t="n">
+      <c r="D22" s="12" t="n">
         <v>1200</v>
       </c>
-      <c r="E22" s="12" t="n">
+      <c r="E22" s="13" t="n">
         <v>45</v>
       </c>
-      <c r="F22" s="11" t="n">
+      <c r="F22" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" s="13" t="n">
+      <c r="G22" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="14" t="n">
         <f aca="false">ROUNDUP((D22*(1+הנחות!$B$6)+E22/60*הנחות!$B$5+F22)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>1630</v>
-      </c>
-      <c r="I22" s="10" t="s">
+        <v>1700</v>
+      </c>
+      <c r="I22" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="J22" s="10" t="s">
+      <c r="J22" s="11" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="D23" s="11" t="n">
+      <c r="D23" s="12" t="n">
         <v>550</v>
       </c>
-      <c r="E23" s="12" t="n">
+      <c r="E23" s="13" t="n">
         <v>45</v>
       </c>
-      <c r="F23" s="11" t="n">
+      <c r="F23" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G23" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H23" s="13" t="n">
+      <c r="G23" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="14" t="n">
         <f aca="false">ROUNDUP((D23*(1+הנחות!$B$6)+E23/60*הנחות!$B$5+F23)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>850</v>
       </c>
-      <c r="I23" s="10" t="s">
+      <c r="I23" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="J23" s="10" t="s">
+      <c r="J23" s="11" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="D24" s="11" t="n">
+      <c r="D24" s="12" t="n">
         <v>120</v>
       </c>
-      <c r="E24" s="12" t="n">
+      <c r="E24" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F24" s="11" t="n">
+      <c r="F24" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G24" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="13" t="n">
+      <c r="G24" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="14" t="n">
         <f aca="false">ROUNDUP((D24*(1+הנחות!$B$6)+E24/60*הנחות!$B$5+F24)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>190</v>
       </c>
-      <c r="I24" s="10" t="s">
+      <c r="I24" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="J24" s="10"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="s">
+      <c r="J24" s="11"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="D25" s="11" t="n">
+      <c r="D25" s="12" t="n">
         <v>70</v>
       </c>
-      <c r="E25" s="12" t="n">
+      <c r="E25" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F25" s="11" t="n">
+      <c r="F25" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H25" s="13" t="n">
+      <c r="G25" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="14" t="n">
         <f aca="false">ROUNDUP((D25*(1+הנחות!$B$6)+E25/60*הנחות!$B$5+F25)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>130</v>
       </c>
-      <c r="I25" s="10" t="s">
+      <c r="I25" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="J25" s="10"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="s">
+      <c r="J25" s="11"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D26" s="11" t="n">
+      <c r="D26" s="12" t="n">
         <v>900</v>
       </c>
-      <c r="E26" s="12" t="n">
+      <c r="E26" s="13" t="n">
         <v>90</v>
       </c>
-      <c r="F26" s="11" t="n">
+      <c r="F26" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G26" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" s="13" t="n">
+      <c r="G26" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="14" t="n">
         <f aca="false">ROUNDUP((D26*(1+הנחות!$B$6)+E26/60*הנחות!$B$5+F26)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>1460</v>
-      </c>
-      <c r="I26" s="10" t="s">
+        <v>1440</v>
+      </c>
+      <c r="I26" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="J26" s="10" t="s">
+      <c r="J26" s="11" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="D27" s="11" t="n">
+      <c r="D27" s="12" t="n">
         <v>330</v>
       </c>
-      <c r="E27" s="12" t="n">
+      <c r="E27" s="13" t="n">
         <v>45</v>
       </c>
-      <c r="F27" s="11" t="n">
+      <c r="F27" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H27" s="13" t="n">
+      <c r="G27" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="14" t="n">
         <f aca="false">ROUNDUP((D27*(1+הנחות!$B$6)+E27/60*הנחות!$B$5+F27)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>590</v>
-      </c>
-      <c r="I27" s="10" t="s">
+        <v>570</v>
+      </c>
+      <c r="I27" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="J27" s="10" t="s">
+      <c r="J27" s="11" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="D28" s="11" t="n">
+      <c r="D28" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="E28" s="12" t="n">
+      <c r="E28" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="F28" s="11" t="n">
+      <c r="F28" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H28" s="13" t="n">
+      <c r="G28" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="14" t="n">
         <f aca="false">ROUNDUP((D28*(1+הנחות!$B$6)+E28/60*הנחות!$B$5+F28)/הנחות!$B$10,0)*הנחות!$B$10</f>
         <v>610</v>
       </c>
-      <c r="I28" s="10" t="s">
+      <c r="I28" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="J28" s="10" t="s">
+      <c r="J28" s="11" t="s">
         <v>109</v>
       </c>
     </row>
@@ -2047,180 +2051,180 @@
   <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="str">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="str">
         <f aca="false">קטלוג!C5</f>
         <v>Home Assistant Green</v>
       </c>
-      <c r="B4" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="16" t="n">
+      <c r="B4" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="17" t="n">
         <f aca="false">קטלוג!H5</f>
-        <v>1080</v>
-      </c>
-      <c r="D4" s="17" t="n">
+        <v>1170</v>
+      </c>
+      <c r="D4" s="18" t="n">
         <f aca="false">B4*C4</f>
-        <v>1080</v>
-      </c>
-      <c r="E4" s="2" t="n">
+        <v>1170</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <f aca="false">B4*קטלוג!G5</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="str">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15" t="str">
         <f aca="false">קטלוג!C6</f>
         <v>מתאם Zigbee/Thread (Connect ZBT / SkyConnect)</v>
       </c>
-      <c r="B5" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="16" t="n">
+      <c r="B5" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="17" t="n">
         <f aca="false">קטלוג!H6</f>
-        <v>300</v>
-      </c>
-      <c r="D5" s="17" t="n">
+        <v>330</v>
+      </c>
+      <c r="D5" s="18" t="n">
         <f aca="false">B5*C5</f>
-        <v>300</v>
-      </c>
-      <c r="E5" s="2" t="n">
+        <v>330</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <f aca="false">B5*קטלוג!G6</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="str">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15" t="str">
         <f aca="false">קטלוג!C12</f>
         <v>חיישן הצפה Aqara</v>
       </c>
-      <c r="B6" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="16" t="n">
+      <c r="B6" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="17" t="n">
         <f aca="false">קטלוג!H12</f>
         <v>150</v>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="D6" s="18" t="n">
         <f aca="false">B6*C6</f>
         <v>150</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="3" t="n">
         <f aca="false">B6*קטלוג!G12</f>
         <v>1</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="str">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="15" t="str">
         <f aca="false">קטלוג!C13</f>
         <v>גלאי עשן Zigbee</v>
       </c>
-      <c r="B7" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="16" t="n">
+      <c r="B7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="17" t="n">
         <f aca="false">קטלוג!H13</f>
         <v>310</v>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D7" s="18" t="n">
         <f aca="false">B7*C7</f>
         <v>310</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <f aca="false">B7*קטלוג!G13</f>
         <v>1</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="15" t="str">
         <f aca="false">קטלוג!C21</f>
         <v>חיישן פתיחה/סגירה (דלת/חלון)</v>
       </c>
-      <c r="B8" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="16" t="n">
+      <c r="B8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="17" t="n">
         <f aca="false">קטלוג!H21</f>
-        <v>140</v>
-      </c>
-      <c r="D8" s="17" t="n">
+        <v>130</v>
+      </c>
+      <c r="D8" s="18" t="n">
         <f aca="false">B8*C8</f>
-        <v>140</v>
-      </c>
-      <c r="E8" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="E8" s="3" t="n">
         <f aca="false">B8*קטלוג!G21</f>
         <v>1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="19" t="n">
         <f aca="false">הנחות!$B$8</f>
         <v>6</v>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C9" s="17" t="n">
         <f aca="false">הנחות!$B$5</f>
-        <v>250</v>
-      </c>
-      <c r="D9" s="17" t="n">
+        <v>180</v>
+      </c>
+      <c r="D9" s="18" t="n">
         <f aca="false">B9*C9</f>
-        <v>1500</v>
-      </c>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
+        <v>1080</v>
+      </c>
+      <c r="E9" s="3"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="19" t="n">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="20" t="n">
         <f aca="false">SUM(D4:D9)</f>
-        <v>3480</v>
-      </c>
-      <c r="E10" s="9" t="n">
+        <v>3170</v>
+      </c>
+      <c r="E10" s="10" t="n">
         <f aca="false">SUM(E4:E8)</f>
         <v>3</v>
       </c>
@@ -2244,94 +2248,94 @@
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="n">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="B4" s="15" t="n">
+      <c r="B4" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="21" t="n">
         <v>160</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="n">
         <v>26</v>
       </c>
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="16" t="n">
         <v>50</v>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="21" t="n">
         <v>220</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="n">
         <v>51</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="21" t="n">
         <v>350</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2352,630 +2356,630 @@
   <dimension ref="A1:G29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="F4" s="21" t="s">
+      <c r="F4" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="G4" s="21" t="s">
+      <c r="G4" s="22" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="str">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15" t="str">
         <f aca="false">קטלוג!C7</f>
         <v>Aqara FP2 (חיישן נוכחות mmWave)</v>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <f aca="false">קטלוג!H7</f>
         <v>610</v>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="17" t="n">
         <f aca="false">קטלוג!F7</f>
         <v>0</v>
       </c>
-      <c r="G5" s="14" t="n">
+      <c r="G5" s="15" t="n">
         <f aca="false">קטלוג!G7</f>
         <v>1</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="str">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15" t="str">
         <f aca="false">קטלוג!C8</f>
         <v>Aqara Motion P1 (PIR למעברים)</v>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="17" t="n">
         <f aca="false">קטלוג!H8</f>
         <v>200</v>
       </c>
-      <c r="C6" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="15" t="n">
+      <c r="C6" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="17" t="n">
         <f aca="false">קטלוג!F8</f>
         <v>0</v>
       </c>
-      <c r="G6" s="14" t="n">
+      <c r="G6" s="15" t="n">
         <f aca="false">קטלוג!G8</f>
         <v>1</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="str">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="15" t="str">
         <f aca="false">קטלוג!C9</f>
         <v>Broadlink RM4 mini (שליטה במזגן IR)</v>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="17" t="n">
         <f aca="false">קטלוג!H9</f>
-        <v>260</v>
-      </c>
-      <c r="C7" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="15" t="n">
+        <v>240</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="16" t="n">
+      <c r="F7" s="17" t="n">
         <f aca="false">קטלוג!F9</f>
         <v>0</v>
       </c>
-      <c r="G7" s="14" t="n">
+      <c r="G7" s="15" t="n">
         <f aca="false">קטלוג!G9</f>
         <v>1</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="15" t="str">
         <f aca="false">קטלוג!C10</f>
         <v>חיישן טמפ'/לחות Aqara</v>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="17" t="n">
         <f aca="false">קטלוג!H10</f>
         <v>150</v>
       </c>
-      <c r="C8" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="15" t="n">
+      <c r="C8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="17" t="n">
         <f aca="false">קטלוג!F10</f>
         <v>0</v>
       </c>
-      <c r="G8" s="14" t="n">
+      <c r="G8" s="15" t="n">
         <f aca="false">קטלוג!G10</f>
         <v>1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="str">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="15" t="str">
         <f aca="false">קטלוג!C11</f>
         <v>IKEA VINDSTYRKA (איכות אוויר)</v>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="17" t="n">
         <f aca="false">קטלוג!H11</f>
         <v>310</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="16" t="n">
+      <c r="D9" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="17" t="n">
         <f aca="false">קטלוג!F11</f>
         <v>0</v>
       </c>
-      <c r="G9" s="14" t="n">
+      <c r="G9" s="15" t="n">
         <f aca="false">קטלוג!G11</f>
         <v>1</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="15" t="str">
         <f aca="false">קטלוג!C12</f>
         <v>חיישן הצפה Aqara</v>
       </c>
-      <c r="B10" s="16" t="n">
+      <c r="B10" s="17" t="n">
         <f aca="false">קטלוג!H12</f>
         <v>150</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="15" t="n">
+      <c r="D10" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="17" t="n">
         <f aca="false">קטלוג!F12</f>
         <v>0</v>
       </c>
-      <c r="G10" s="14" t="n">
+      <c r="G10" s="15" t="n">
         <f aca="false">קטלוג!G12</f>
         <v>1</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="str">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="15" t="str">
         <f aca="false">קטלוג!C14</f>
         <v>Shelly Pro 1PM DIN-Rail (ניתוק אוטומטי בלוח)</v>
       </c>
-      <c r="B11" s="16" t="n">
+      <c r="B11" s="17" t="n">
         <f aca="false">קטלוג!H14</f>
-        <v>810</v>
-      </c>
-      <c r="C11" s="15" t="n">
+        <v>820</v>
+      </c>
+      <c r="C11" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="16" t="n">
+      <c r="D11" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="17" t="n">
         <f aca="false">קטלוג!F14</f>
         <v>300</v>
       </c>
-      <c r="G11" s="14" t="n">
+      <c r="G11" s="15" t="n">
         <f aca="false">קטלוג!G14</f>
         <v>1</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="str">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="15" t="str">
         <f aca="false">קטלוג!C15</f>
         <v>Switcher (בקרת דוד)</v>
       </c>
-      <c r="B12" s="16" t="n">
+      <c r="B12" s="17" t="n">
         <f aca="false">קטלוג!H15</f>
-        <v>790</v>
-      </c>
-      <c r="C12" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="16" t="n">
+        <v>810</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="17" t="n">
         <f aca="false">קטלוג!F15</f>
         <v>250</v>
       </c>
-      <c r="G12" s="14" t="n">
+      <c r="G12" s="15" t="n">
         <f aca="false">קטלוג!G15</f>
         <v>1</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="str">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="15" t="str">
         <f aca="false">קטלוג!C16</f>
         <v>Shelly EM (מדידה חד-פאזית)</v>
       </c>
-      <c r="B13" s="16" t="n">
+      <c r="B13" s="17" t="n">
         <f aca="false">קטלוג!H16</f>
-        <v>680</v>
-      </c>
-      <c r="C13" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="15" t="n">
+        <v>690</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="16" t="n">
+      <c r="F13" s="17" t="n">
         <f aca="false">קטלוג!F16</f>
         <v>250</v>
       </c>
-      <c r="G13" s="14" t="n">
+      <c r="G13" s="15" t="n">
         <f aca="false">קטלוג!G16</f>
         <v>1</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="str">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="15" t="str">
         <f aca="false">קטלוג!C17</f>
         <v>Shelly Pro 3EM (מדידה תלת-פאזית)</v>
       </c>
-      <c r="B14" s="16" t="n">
+      <c r="B14" s="17" t="n">
         <f aca="false">קטלוג!H17</f>
-        <v>1220</v>
-      </c>
-      <c r="C14" s="15" t="n">
+        <v>1260</v>
+      </c>
+      <c r="C14" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="16" t="n">
+      <c r="E14" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="17" t="n">
         <f aca="false">קטלוג!F17</f>
         <v>350</v>
       </c>
-      <c r="G14" s="14" t="n">
+      <c r="G14" s="15" t="n">
         <f aca="false">קטלוג!G17</f>
         <v>1</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14" t="str">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="15" t="str">
         <f aca="false">קטלוג!C18</f>
         <v>Shelly 1PM (מתג תאורה, לכל נקודה)</v>
       </c>
-      <c r="B15" s="16" t="n">
+      <c r="B15" s="17" t="n">
         <f aca="false">קטלוג!H18</f>
         <v>330</v>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="D15" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="E15" s="15" t="n">
+      <c r="E15" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="F15" s="16" t="n">
+      <c r="F15" s="17" t="n">
         <f aca="false">קטלוג!F18</f>
         <v>150</v>
       </c>
-      <c r="G15" s="14" t="n">
+      <c r="G15" s="15" t="n">
         <f aca="false">קטלוג!G18</f>
         <v>1</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="str">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="15" t="str">
         <f aca="false">קטלוג!C19</f>
         <v>Shelly 2PM (תריס חשמלי)</v>
       </c>
-      <c r="B16" s="16" t="n">
+      <c r="B16" s="17" t="n">
         <f aca="false">קטלוג!H19</f>
         <v>410</v>
       </c>
-      <c r="C16" s="15" t="n">
+      <c r="C16" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="15" t="n">
+      <c r="D16" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="15" t="n">
+      <c r="E16" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="F16" s="16" t="n">
+      <c r="F16" s="17" t="n">
         <f aca="false">קטלוג!F19</f>
         <v>150</v>
       </c>
-      <c r="G16" s="14" t="n">
+      <c r="G16" s="15" t="n">
         <f aca="false">קטלוג!G19</f>
         <v>1</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="str">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="15" t="str">
         <f aca="false">קטלוג!C20</f>
         <v>Shelly Dimmer (עמעם)</v>
       </c>
-      <c r="B17" s="16" t="n">
+      <c r="B17" s="17" t="n">
         <f aca="false">קטלוג!H20</f>
-        <v>400</v>
-      </c>
-      <c r="C17" s="15" t="n">
+        <v>410</v>
+      </c>
+      <c r="C17" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="15" t="n">
+      <c r="D17" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="15" t="n">
+      <c r="E17" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="16" t="n">
+      <c r="F17" s="17" t="n">
         <f aca="false">קטלוג!F20</f>
         <v>150</v>
       </c>
-      <c r="G17" s="14" t="n">
+      <c r="G17" s="15" t="n">
         <f aca="false">קטלוג!G20</f>
         <v>1</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="str">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="15" t="str">
         <f aca="false">קטלוג!C21</f>
         <v>חיישן פתיחה/סגירה (דלת/חלון)</v>
       </c>
-      <c r="B18" s="16" t="n">
+      <c r="B18" s="17" t="n">
         <f aca="false">קטלוג!H21</f>
-        <v>140</v>
-      </c>
-      <c r="C18" s="15" t="n">
+        <v>130</v>
+      </c>
+      <c r="C18" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="D18" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="E18" s="15" t="n">
+      <c r="E18" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="16" t="n">
+      <c r="F18" s="17" t="n">
         <f aca="false">קטלוג!F21</f>
         <v>0</v>
       </c>
-      <c r="G18" s="14" t="n">
+      <c r="G18" s="15" t="n">
         <f aca="false">קטלוג!G21</f>
         <v>1</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B20" s="2"/>
-      <c r="C20" s="22" t="n">
+      <c r="B20" s="3"/>
+      <c r="C20" s="23" t="n">
         <f aca="false">SUMPRODUCT($B$5:$B$18,C5:C18)</f>
-        <v>4850</v>
-      </c>
-      <c r="D20" s="22" t="n">
+        <v>4820</v>
+      </c>
+      <c r="D20" s="23" t="n">
         <f aca="false">SUMPRODUCT($B$5:$B$18,D5:D18)</f>
-        <v>10240</v>
-      </c>
-      <c r="E20" s="22" t="n">
+        <v>10210</v>
+      </c>
+      <c r="E20" s="23" t="n">
         <f aca="false">SUMPRODUCT($B$5:$B$18,E5:E18)</f>
-        <v>17340</v>
-      </c>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
+        <v>17290</v>
+      </c>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="22" t="n">
+      <c r="B21" s="3"/>
+      <c r="C21" s="23" t="n">
         <f aca="false">'חבילה בסיסית'!$D$10</f>
-        <v>3480</v>
-      </c>
-      <c r="D21" s="22" t="n">
+        <v>3170</v>
+      </c>
+      <c r="D21" s="23" t="n">
         <f aca="false">'חבילה בסיסית'!$D$10</f>
-        <v>3480</v>
-      </c>
-      <c r="E21" s="22" t="n">
+        <v>3170</v>
+      </c>
+      <c r="E21" s="23" t="n">
         <f aca="false">'חבילה בסיסית'!$D$10</f>
-        <v>3480</v>
-      </c>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
+        <v>3170</v>
+      </c>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="22" t="n">
+      <c r="B22" s="3"/>
+      <c r="C22" s="23" t="n">
         <f aca="false">IF(SUMPRODUCT(($F$5:$F$18&gt;0)*C5:C18)&gt;0,הנחות!$B$7,0)</f>
-        <v>400</v>
-      </c>
-      <c r="D22" s="22" t="n">
+        <v>495</v>
+      </c>
+      <c r="D22" s="23" t="n">
         <f aca="false">IF(SUMPRODUCT(($F$5:$F$18&gt;0)*D5:D18)&gt;0,הנחות!$B$7,0)</f>
-        <v>400</v>
-      </c>
-      <c r="E22" s="22" t="n">
+        <v>495</v>
+      </c>
+      <c r="E22" s="23" t="n">
         <f aca="false">IF(SUMPRODUCT(($F$5:$F$18&gt;0)*E5:E18)&gt;0,הנחות!$B$7,0)</f>
-        <v>400</v>
-      </c>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="s">
+        <v>495</v>
+      </c>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="19" t="n">
+      <c r="B23" s="3"/>
+      <c r="C23" s="20" t="n">
         <f aca="false">SUM(C20:C22)</f>
-        <v>8730</v>
-      </c>
-      <c r="D23" s="19" t="n">
+        <v>8485</v>
+      </c>
+      <c r="D23" s="20" t="n">
         <f aca="false">SUM(D20:D22)</f>
-        <v>14120</v>
-      </c>
-      <c r="E23" s="19" t="n">
+        <v>13875</v>
+      </c>
+      <c r="E23" s="20" t="n">
         <f aca="false">SUM(E20:E22)</f>
-        <v>21220</v>
-      </c>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="s">
+        <v>20955</v>
+      </c>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="23" t="n">
+      <c r="B24" s="3"/>
+      <c r="C24" s="24" t="n">
         <v>5700</v>
       </c>
-      <c r="D24" s="23" t="n">
+      <c r="D24" s="24" t="n">
         <v>8700</v>
       </c>
-      <c r="E24" s="23" t="n">
+      <c r="E24" s="24" t="n">
         <v>13150</v>
       </c>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="9" t="s">
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="22" t="n">
+      <c r="B25" s="3"/>
+      <c r="C25" s="23" t="n">
         <f aca="false">C23-C24</f>
-        <v>3030</v>
-      </c>
-      <c r="D25" s="22" t="n">
+        <v>2785</v>
+      </c>
+      <c r="D25" s="23" t="n">
         <f aca="false">D23-D24</f>
-        <v>5420</v>
-      </c>
-      <c r="E25" s="22" t="n">
+        <v>5175</v>
+      </c>
+      <c r="E25" s="23" t="n">
         <f aca="false">E23-E24</f>
-        <v>8070</v>
-      </c>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
+        <v>7805</v>
+      </c>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="24" t="n">
+      <c r="B26" s="3"/>
+      <c r="C26" s="25" t="n">
         <f aca="false">'חבילה בסיסית'!$E$10+SUMPRODUCT($G$5:$G$18,C5:C18)</f>
         <v>17</v>
       </c>
-      <c r="D26" s="24" t="n">
+      <c r="D26" s="25" t="n">
         <f aca="false">'חבילה בסיסית'!$E$10+SUMPRODUCT($G$5:$G$18,D5:D18)</f>
         <v>32</v>
       </c>
-      <c r="E26" s="24" t="n">
+      <c r="E26" s="25" t="n">
         <f aca="false">'חבילה בסיסית'!$E$10+SUMPRODUCT($G$5:$G$18,E5:E18)</f>
         <v>54</v>
       </c>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="9" t="s">
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="22" t="n">
+      <c r="B27" s="3"/>
+      <c r="C27" s="23" t="n">
         <f aca="false">INDEX(ריטיינר!$C$4:$C$6,MATCH(C26,ריטיינר!$A$4:$A$6,1))</f>
         <v>160</v>
       </c>
-      <c r="D27" s="22" t="n">
+      <c r="D27" s="23" t="n">
         <f aca="false">INDEX(ריטיינר!$C$4:$C$6,MATCH(D26,ריטיינר!$A$4:$A$6,1))</f>
         <v>220</v>
       </c>
-      <c r="E27" s="22" t="n">
+      <c r="E27" s="23" t="n">
         <f aca="false">INDEX(ריטיינר!$C$4:$C$6,MATCH(E26,ריטיינר!$A$4:$A$6,1))</f>
         <v>350</v>
       </c>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2996,1018 +3000,1018 @@
   <dimension ref="A1:G52"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="25" t="n">
+      <c r="D5" s="26" t="n">
         <f aca="false">IF(B5="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B5,קטלוג!$C$5:$C$28,0)))</f>
         <v>330</v>
       </c>
-      <c r="E5" s="25" t="n">
+      <c r="E5" s="26" t="n">
         <f aca="false">IF(B5="","",C5*D5)</f>
         <v>990</v>
       </c>
-      <c r="F5" s="26" t="n">
+      <c r="F5" s="27" t="n">
         <f aca="false">IF(B5="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B5,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v>1</v>
       </c>
-      <c r="G5" s="26" t="n">
+      <c r="G5" s="27" t="n">
         <f aca="false">IF(B5="","",C5*INDEX(קטלוג!$G$5:$G$28,MATCH(B5,קטלוג!$C$5:$C$28,0)))</f>
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="25" t="str">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="26" t="str">
         <f aca="false">IF(B6="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B6,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E6" s="25" t="str">
+      <c r="E6" s="26" t="str">
         <f aca="false">IF(B6="","",C6*D6)</f>
         <v/>
       </c>
-      <c r="F6" s="26" t="str">
+      <c r="F6" s="27" t="str">
         <f aca="false">IF(B6="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B6,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G6" s="26" t="str">
+      <c r="G6" s="27" t="str">
         <f aca="false">IF(B6="","",C6*INDEX(קטלוג!$G$5:$G$28,MATCH(B6,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="25" t="str">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="26" t="str">
         <f aca="false">IF(B7="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B7,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E7" s="25" t="str">
+      <c r="E7" s="26" t="str">
         <f aca="false">IF(B7="","",C7*D7)</f>
         <v/>
       </c>
-      <c r="F7" s="26" t="str">
+      <c r="F7" s="27" t="str">
         <f aca="false">IF(B7="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B7,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G7" s="26" t="str">
+      <c r="G7" s="27" t="str">
         <f aca="false">IF(B7="","",C7*INDEX(קטלוג!$G$5:$G$28,MATCH(B7,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="25" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="26" t="str">
         <f aca="false">IF(B8="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B8,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E8" s="25" t="str">
+      <c r="E8" s="26" t="str">
         <f aca="false">IF(B8="","",C8*D8)</f>
         <v/>
       </c>
-      <c r="F8" s="26" t="str">
+      <c r="F8" s="27" t="str">
         <f aca="false">IF(B8="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B8,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G8" s="26" t="str">
+      <c r="G8" s="27" t="str">
         <f aca="false">IF(B8="","",C8*INDEX(קטלוג!$G$5:$G$28,MATCH(B8,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="25" t="str">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="26" t="str">
         <f aca="false">IF(B9="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B9,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E9" s="25" t="str">
+      <c r="E9" s="26" t="str">
         <f aca="false">IF(B9="","",C9*D9)</f>
         <v/>
       </c>
-      <c r="F9" s="26" t="str">
+      <c r="F9" s="27" t="str">
         <f aca="false">IF(B9="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B9,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G9" s="26" t="str">
+      <c r="G9" s="27" t="str">
         <f aca="false">IF(B9="","",C9*INDEX(קטלוג!$G$5:$G$28,MATCH(B9,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="25" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="26" t="str">
         <f aca="false">IF(B10="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B10,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E10" s="25" t="str">
+      <c r="E10" s="26" t="str">
         <f aca="false">IF(B10="","",C10*D10)</f>
         <v/>
       </c>
-      <c r="F10" s="26" t="str">
+      <c r="F10" s="27" t="str">
         <f aca="false">IF(B10="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B10,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G10" s="26" t="str">
+      <c r="G10" s="27" t="str">
         <f aca="false">IF(B10="","",C10*INDEX(קטלוג!$G$5:$G$28,MATCH(B10,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="25" t="str">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="26" t="str">
         <f aca="false">IF(B11="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B11,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E11" s="25" t="str">
+      <c r="E11" s="26" t="str">
         <f aca="false">IF(B11="","",C11*D11)</f>
         <v/>
       </c>
-      <c r="F11" s="26" t="str">
+      <c r="F11" s="27" t="str">
         <f aca="false">IF(B11="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B11,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G11" s="26" t="str">
+      <c r="G11" s="27" t="str">
         <f aca="false">IF(B11="","",C11*INDEX(קטלוג!$G$5:$G$28,MATCH(B11,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="25" t="str">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="26" t="str">
         <f aca="false">IF(B12="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B12,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E12" s="25" t="str">
+      <c r="E12" s="26" t="str">
         <f aca="false">IF(B12="","",C12*D12)</f>
         <v/>
       </c>
-      <c r="F12" s="26" t="str">
+      <c r="F12" s="27" t="str">
         <f aca="false">IF(B12="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B12,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G12" s="26" t="str">
+      <c r="G12" s="27" t="str">
         <f aca="false">IF(B12="","",C12*INDEX(קטלוג!$G$5:$G$28,MATCH(B12,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="25" t="str">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="26" t="str">
         <f aca="false">IF(B13="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B13,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E13" s="25" t="str">
+      <c r="E13" s="26" t="str">
         <f aca="false">IF(B13="","",C13*D13)</f>
         <v/>
       </c>
-      <c r="F13" s="26" t="str">
+      <c r="F13" s="27" t="str">
         <f aca="false">IF(B13="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B13,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G13" s="26" t="str">
+      <c r="G13" s="27" t="str">
         <f aca="false">IF(B13="","",C13*INDEX(קטלוג!$G$5:$G$28,MATCH(B13,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="25" t="str">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="26" t="str">
         <f aca="false">IF(B14="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B14,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E14" s="25" t="str">
+      <c r="E14" s="26" t="str">
         <f aca="false">IF(B14="","",C14*D14)</f>
         <v/>
       </c>
-      <c r="F14" s="26" t="str">
+      <c r="F14" s="27" t="str">
         <f aca="false">IF(B14="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B14,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G14" s="26" t="str">
+      <c r="G14" s="27" t="str">
         <f aca="false">IF(B14="","",C14*INDEX(קטלוג!$G$5:$G$28,MATCH(B14,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="25" t="str">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="26" t="str">
         <f aca="false">IF(B15="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B15,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E15" s="25" t="str">
+      <c r="E15" s="26" t="str">
         <f aca="false">IF(B15="","",C15*D15)</f>
         <v/>
       </c>
-      <c r="F15" s="26" t="str">
+      <c r="F15" s="27" t="str">
         <f aca="false">IF(B15="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B15,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G15" s="26" t="str">
+      <c r="G15" s="27" t="str">
         <f aca="false">IF(B15="","",C15*INDEX(קטלוג!$G$5:$G$28,MATCH(B15,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="25" t="str">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="26" t="str">
         <f aca="false">IF(B16="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B16,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E16" s="25" t="str">
+      <c r="E16" s="26" t="str">
         <f aca="false">IF(B16="","",C16*D16)</f>
         <v/>
       </c>
-      <c r="F16" s="26" t="str">
+      <c r="F16" s="27" t="str">
         <f aca="false">IF(B16="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B16,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G16" s="26" t="str">
+      <c r="G16" s="27" t="str">
         <f aca="false">IF(B16="","",C16*INDEX(קטלוג!$G$5:$G$28,MATCH(B16,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="25" t="str">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="26" t="str">
         <f aca="false">IF(B17="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B17,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E17" s="25" t="str">
+      <c r="E17" s="26" t="str">
         <f aca="false">IF(B17="","",C17*D17)</f>
         <v/>
       </c>
-      <c r="F17" s="26" t="str">
+      <c r="F17" s="27" t="str">
         <f aca="false">IF(B17="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B17,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G17" s="26" t="str">
+      <c r="G17" s="27" t="str">
         <f aca="false">IF(B17="","",C17*INDEX(קטלוג!$G$5:$G$28,MATCH(B17,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="25" t="str">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="26" t="str">
         <f aca="false">IF(B18="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B18,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E18" s="25" t="str">
+      <c r="E18" s="26" t="str">
         <f aca="false">IF(B18="","",C18*D18)</f>
         <v/>
       </c>
-      <c r="F18" s="26" t="str">
+      <c r="F18" s="27" t="str">
         <f aca="false">IF(B18="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B18,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G18" s="26" t="str">
+      <c r="G18" s="27" t="str">
         <f aca="false">IF(B18="","",C18*INDEX(קטלוג!$G$5:$G$28,MATCH(B18,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="25" t="str">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="26" t="str">
         <f aca="false">IF(B19="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B19,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E19" s="25" t="str">
+      <c r="E19" s="26" t="str">
         <f aca="false">IF(B19="","",C19*D19)</f>
         <v/>
       </c>
-      <c r="F19" s="26" t="str">
+      <c r="F19" s="27" t="str">
         <f aca="false">IF(B19="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B19,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G19" s="26" t="str">
+      <c r="G19" s="27" t="str">
         <f aca="false">IF(B19="","",C19*INDEX(קטלוג!$G$5:$G$28,MATCH(B19,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="25" t="str">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="26" t="str">
         <f aca="false">IF(B20="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B20,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E20" s="25" t="str">
+      <c r="E20" s="26" t="str">
         <f aca="false">IF(B20="","",C20*D20)</f>
         <v/>
       </c>
-      <c r="F20" s="26" t="str">
+      <c r="F20" s="27" t="str">
         <f aca="false">IF(B20="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B20,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G20" s="26" t="str">
+      <c r="G20" s="27" t="str">
         <f aca="false">IF(B20="","",C20*INDEX(קטלוג!$G$5:$G$28,MATCH(B20,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="25" t="str">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="26" t="str">
         <f aca="false">IF(B21="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B21,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E21" s="25" t="str">
+      <c r="E21" s="26" t="str">
         <f aca="false">IF(B21="","",C21*D21)</f>
         <v/>
       </c>
-      <c r="F21" s="26" t="str">
+      <c r="F21" s="27" t="str">
         <f aca="false">IF(B21="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B21,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G21" s="26" t="str">
+      <c r="G21" s="27" t="str">
         <f aca="false">IF(B21="","",C21*INDEX(קטלוג!$G$5:$G$28,MATCH(B21,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="25" t="str">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="26" t="str">
         <f aca="false">IF(B22="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B22,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E22" s="25" t="str">
+      <c r="E22" s="26" t="str">
         <f aca="false">IF(B22="","",C22*D22)</f>
         <v/>
       </c>
-      <c r="F22" s="26" t="str">
+      <c r="F22" s="27" t="str">
         <f aca="false">IF(B22="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B22,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G22" s="26" t="str">
+      <c r="G22" s="27" t="str">
         <f aca="false">IF(B22="","",C22*INDEX(קטלוג!$G$5:$G$28,MATCH(B22,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="25" t="str">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="26" t="str">
         <f aca="false">IF(B23="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B23,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E23" s="25" t="str">
+      <c r="E23" s="26" t="str">
         <f aca="false">IF(B23="","",C23*D23)</f>
         <v/>
       </c>
-      <c r="F23" s="26" t="str">
+      <c r="F23" s="27" t="str">
         <f aca="false">IF(B23="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B23,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G23" s="26" t="str">
+      <c r="G23" s="27" t="str">
         <f aca="false">IF(B23="","",C23*INDEX(קטלוג!$G$5:$G$28,MATCH(B23,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="25" t="str">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="26" t="str">
         <f aca="false">IF(B24="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B24,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E24" s="25" t="str">
+      <c r="E24" s="26" t="str">
         <f aca="false">IF(B24="","",C24*D24)</f>
         <v/>
       </c>
-      <c r="F24" s="26" t="str">
+      <c r="F24" s="27" t="str">
         <f aca="false">IF(B24="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B24,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G24" s="26" t="str">
+      <c r="G24" s="27" t="str">
         <f aca="false">IF(B24="","",C24*INDEX(קטלוג!$G$5:$G$28,MATCH(B24,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="25" t="str">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="26" t="str">
         <f aca="false">IF(B25="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B25,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E25" s="25" t="str">
+      <c r="E25" s="26" t="str">
         <f aca="false">IF(B25="","",C25*D25)</f>
         <v/>
       </c>
-      <c r="F25" s="26" t="str">
+      <c r="F25" s="27" t="str">
         <f aca="false">IF(B25="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B25,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G25" s="26" t="str">
+      <c r="G25" s="27" t="str">
         <f aca="false">IF(B25="","",C25*INDEX(קטלוג!$G$5:$G$28,MATCH(B25,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="12"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="25" t="str">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="26" t="str">
         <f aca="false">IF(B26="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B26,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E26" s="25" t="str">
+      <c r="E26" s="26" t="str">
         <f aca="false">IF(B26="","",C26*D26)</f>
         <v/>
       </c>
-      <c r="F26" s="26" t="str">
+      <c r="F26" s="27" t="str">
         <f aca="false">IF(B26="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B26,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G26" s="26" t="str">
+      <c r="G26" s="27" t="str">
         <f aca="false">IF(B26="","",C26*INDEX(קטלוג!$G$5:$G$28,MATCH(B26,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="25" t="str">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="26" t="str">
         <f aca="false">IF(B27="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B27,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E27" s="25" t="str">
+      <c r="E27" s="26" t="str">
         <f aca="false">IF(B27="","",C27*D27)</f>
         <v/>
       </c>
-      <c r="F27" s="26" t="str">
+      <c r="F27" s="27" t="str">
         <f aca="false">IF(B27="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B27,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G27" s="26" t="str">
+      <c r="G27" s="27" t="str">
         <f aca="false">IF(B27="","",C27*INDEX(קטלוג!$G$5:$G$28,MATCH(B27,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="25" t="str">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="26" t="str">
         <f aca="false">IF(B28="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B28,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E28" s="25" t="str">
+      <c r="E28" s="26" t="str">
         <f aca="false">IF(B28="","",C28*D28)</f>
         <v/>
       </c>
-      <c r="F28" s="26" t="str">
+      <c r="F28" s="27" t="str">
         <f aca="false">IF(B28="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B28,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G28" s="26" t="str">
+      <c r="G28" s="27" t="str">
         <f aca="false">IF(B28="","",C28*INDEX(קטלוג!$G$5:$G$28,MATCH(B28,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="25" t="str">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="13"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="26" t="str">
         <f aca="false">IF(B29="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B29,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E29" s="25" t="str">
+      <c r="E29" s="26" t="str">
         <f aca="false">IF(B29="","",C29*D29)</f>
         <v/>
       </c>
-      <c r="F29" s="26" t="str">
+      <c r="F29" s="27" t="str">
         <f aca="false">IF(B29="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B29,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G29" s="26" t="str">
+      <c r="G29" s="27" t="str">
         <f aca="false">IF(B29="","",C29*INDEX(קטלוג!$G$5:$G$28,MATCH(B29,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="12"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="25" t="str">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="26" t="str">
         <f aca="false">IF(B30="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B30,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E30" s="25" t="str">
+      <c r="E30" s="26" t="str">
         <f aca="false">IF(B30="","",C30*D30)</f>
         <v/>
       </c>
-      <c r="F30" s="26" t="str">
+      <c r="F30" s="27" t="str">
         <f aca="false">IF(B30="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B30,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G30" s="26" t="str">
+      <c r="G30" s="27" t="str">
         <f aca="false">IF(B30="","",C30*INDEX(קטלוג!$G$5:$G$28,MATCH(B30,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="25" t="str">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="26" t="str">
         <f aca="false">IF(B31="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B31,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E31" s="25" t="str">
+      <c r="E31" s="26" t="str">
         <f aca="false">IF(B31="","",C31*D31)</f>
         <v/>
       </c>
-      <c r="F31" s="26" t="str">
+      <c r="F31" s="27" t="str">
         <f aca="false">IF(B31="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B31,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G31" s="26" t="str">
+      <c r="G31" s="27" t="str">
         <f aca="false">IF(B31="","",C31*INDEX(קטלוג!$G$5:$G$28,MATCH(B31,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="12"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="25" t="str">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="26" t="str">
         <f aca="false">IF(B32="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B32,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E32" s="25" t="str">
+      <c r="E32" s="26" t="str">
         <f aca="false">IF(B32="","",C32*D32)</f>
         <v/>
       </c>
-      <c r="F32" s="26" t="str">
+      <c r="F32" s="27" t="str">
         <f aca="false">IF(B32="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B32,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G32" s="26" t="str">
+      <c r="G32" s="27" t="str">
         <f aca="false">IF(B32="","",C32*INDEX(קטלוג!$G$5:$G$28,MATCH(B32,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="12"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="25" t="str">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="26" t="str">
         <f aca="false">IF(B33="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B33,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E33" s="25" t="str">
+      <c r="E33" s="26" t="str">
         <f aca="false">IF(B33="","",C33*D33)</f>
         <v/>
       </c>
-      <c r="F33" s="26" t="str">
+      <c r="F33" s="27" t="str">
         <f aca="false">IF(B33="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B33,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G33" s="26" t="str">
+      <c r="G33" s="27" t="str">
         <f aca="false">IF(B33="","",C33*INDEX(קטלוג!$G$5:$G$28,MATCH(B33,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="12"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="25" t="str">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="26" t="str">
         <f aca="false">IF(B34="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B34,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E34" s="25" t="str">
+      <c r="E34" s="26" t="str">
         <f aca="false">IF(B34="","",C34*D34)</f>
         <v/>
       </c>
-      <c r="F34" s="26" t="str">
+      <c r="F34" s="27" t="str">
         <f aca="false">IF(B34="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B34,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G34" s="26" t="str">
+      <c r="G34" s="27" t="str">
         <f aca="false">IF(B34="","",C34*INDEX(קטלוג!$G$5:$G$28,MATCH(B34,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12"/>
-      <c r="B35" s="12"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="25" t="str">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="13"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="26" t="str">
         <f aca="false">IF(B35="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B35,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E35" s="25" t="str">
+      <c r="E35" s="26" t="str">
         <f aca="false">IF(B35="","",C35*D35)</f>
         <v/>
       </c>
-      <c r="F35" s="26" t="str">
+      <c r="F35" s="27" t="str">
         <f aca="false">IF(B35="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B35,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G35" s="26" t="str">
+      <c r="G35" s="27" t="str">
         <f aca="false">IF(B35="","",C35*INDEX(קטלוג!$G$5:$G$28,MATCH(B35,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12"/>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="25" t="str">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="13"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="26" t="str">
         <f aca="false">IF(B36="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B36,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E36" s="25" t="str">
+      <c r="E36" s="26" t="str">
         <f aca="false">IF(B36="","",C36*D36)</f>
         <v/>
       </c>
-      <c r="F36" s="26" t="str">
+      <c r="F36" s="27" t="str">
         <f aca="false">IF(B36="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B36,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G36" s="26" t="str">
+      <c r="G36" s="27" t="str">
         <f aca="false">IF(B36="","",C36*INDEX(קטלוג!$G$5:$G$28,MATCH(B36,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="12"/>
-      <c r="B37" s="12"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="25" t="str">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="26" t="str">
         <f aca="false">IF(B37="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B37,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E37" s="25" t="str">
+      <c r="E37" s="26" t="str">
         <f aca="false">IF(B37="","",C37*D37)</f>
         <v/>
       </c>
-      <c r="F37" s="26" t="str">
+      <c r="F37" s="27" t="str">
         <f aca="false">IF(B37="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B37,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G37" s="26" t="str">
+      <c r="G37" s="27" t="str">
         <f aca="false">IF(B37="","",C37*INDEX(קטלוג!$G$5:$G$28,MATCH(B37,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12"/>
-      <c r="B38" s="12"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="25" t="str">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="26" t="str">
         <f aca="false">IF(B38="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B38,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E38" s="25" t="str">
+      <c r="E38" s="26" t="str">
         <f aca="false">IF(B38="","",C38*D38)</f>
         <v/>
       </c>
-      <c r="F38" s="26" t="str">
+      <c r="F38" s="27" t="str">
         <f aca="false">IF(B38="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B38,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G38" s="26" t="str">
+      <c r="G38" s="27" t="str">
         <f aca="false">IF(B38="","",C38*INDEX(קטלוג!$G$5:$G$28,MATCH(B38,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="12"/>
-      <c r="B39" s="12"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="25" t="str">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="26" t="str">
         <f aca="false">IF(B39="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B39,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E39" s="25" t="str">
+      <c r="E39" s="26" t="str">
         <f aca="false">IF(B39="","",C39*D39)</f>
         <v/>
       </c>
-      <c r="F39" s="26" t="str">
+      <c r="F39" s="27" t="str">
         <f aca="false">IF(B39="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B39,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G39" s="26" t="str">
+      <c r="G39" s="27" t="str">
         <f aca="false">IF(B39="","",C39*INDEX(קטלוג!$G$5:$G$28,MATCH(B39,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="12"/>
-      <c r="B40" s="12"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="25" t="str">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="13"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="26" t="str">
         <f aca="false">IF(B40="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B40,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E40" s="25" t="str">
+      <c r="E40" s="26" t="str">
         <f aca="false">IF(B40="","",C40*D40)</f>
         <v/>
       </c>
-      <c r="F40" s="26" t="str">
+      <c r="F40" s="27" t="str">
         <f aca="false">IF(B40="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B40,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G40" s="26" t="str">
+      <c r="G40" s="27" t="str">
         <f aca="false">IF(B40="","",C40*INDEX(קטלוג!$G$5:$G$28,MATCH(B40,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="12"/>
-      <c r="B41" s="12"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="25" t="str">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="13"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="26" t="str">
         <f aca="false">IF(B41="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B41,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E41" s="25" t="str">
+      <c r="E41" s="26" t="str">
         <f aca="false">IF(B41="","",C41*D41)</f>
         <v/>
       </c>
-      <c r="F41" s="26" t="str">
+      <c r="F41" s="27" t="str">
         <f aca="false">IF(B41="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B41,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G41" s="26" t="str">
+      <c r="G41" s="27" t="str">
         <f aca="false">IF(B41="","",C41*INDEX(קטלוג!$G$5:$G$28,MATCH(B41,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="12"/>
-      <c r="B42" s="12"/>
-      <c r="C42" s="12"/>
-      <c r="D42" s="25" t="str">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13"/>
+      <c r="B42" s="13"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="26" t="str">
         <f aca="false">IF(B42="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B42,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E42" s="25" t="str">
+      <c r="E42" s="26" t="str">
         <f aca="false">IF(B42="","",C42*D42)</f>
         <v/>
       </c>
-      <c r="F42" s="26" t="str">
+      <c r="F42" s="27" t="str">
         <f aca="false">IF(B42="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B42,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G42" s="26" t="str">
+      <c r="G42" s="27" t="str">
         <f aca="false">IF(B42="","",C42*INDEX(קטלוג!$G$5:$G$28,MATCH(B42,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="12"/>
-      <c r="B43" s="12"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="25" t="str">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13"/>
+      <c r="B43" s="13"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="26" t="str">
         <f aca="false">IF(B43="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B43,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E43" s="25" t="str">
+      <c r="E43" s="26" t="str">
         <f aca="false">IF(B43="","",C43*D43)</f>
         <v/>
       </c>
-      <c r="F43" s="26" t="str">
+      <c r="F43" s="27" t="str">
         <f aca="false">IF(B43="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B43,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G43" s="26" t="str">
+      <c r="G43" s="27" t="str">
         <f aca="false">IF(B43="","",C43*INDEX(קטלוג!$G$5:$G$28,MATCH(B43,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="12"/>
-      <c r="B44" s="12"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="25" t="str">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="13"/>
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="26" t="str">
         <f aca="false">IF(B44="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B44,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
-      <c r="E44" s="25" t="str">
+      <c r="E44" s="26" t="str">
         <f aca="false">IF(B44="","",C44*D44)</f>
         <v/>
       </c>
-      <c r="F44" s="26" t="str">
+      <c r="F44" s="27" t="str">
         <f aca="false">IF(B44="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B44,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
         <v/>
       </c>
-      <c r="G44" s="26" t="str">
+      <c r="G44" s="27" t="str">
         <f aca="false">IF(B44="","",C44*INDEX(קטלוג!$G$5:$G$28,MATCH(B44,קטלוג!$C$5:$C$28,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="9" t="s">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="3"/>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="B46" s="17" t="n">
+      <c r="B46" s="18" t="n">
         <f aca="false">SUM(E5:E44)</f>
         <v>990</v>
       </c>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="2"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="9" t="s">
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="B47" s="17" t="n">
+      <c r="B47" s="18" t="n">
         <f aca="false">'חבילה בסיסית'!$D$10</f>
-        <v>3480</v>
-      </c>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="9" t="s">
+        <v>3170</v>
+      </c>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B48" s="17" t="n">
+      <c r="B48" s="18" t="n">
         <f aca="false">IF(SUMPRODUCT((F5:F44=1)*1)&gt;0,הנחות!$B$7,0)</f>
-        <v>400</v>
-      </c>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="2"/>
-      <c r="G48" s="2"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="9" t="s">
+        <v>495</v>
+      </c>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="B49" s="19" t="n">
+      <c r="B49" s="20" t="n">
         <f aca="false">SUM(B46:B48)</f>
-        <v>4870</v>
-      </c>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-      <c r="G49" s="2"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="9" t="s">
+        <v>4655</v>
+      </c>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="B50" s="27" t="n">
+      <c r="B50" s="28" t="n">
         <f aca="false">'חבילה בסיסית'!$E$10+SUM(G5:G44)</f>
         <v>6</v>
       </c>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-      <c r="G50" s="2"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="9" t="s">
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="B51" s="19" t="n">
+      <c r="B51" s="20" t="n">
         <f aca="false">INDEX(ריטיינר!$C$4:$C$6,MATCH(B50,ריטיינר!$A$4:$A$6,1))</f>
         <v>160</v>
       </c>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Verify hardware prices against Israeli importers; slim starting points (FP300, Shelly boiler kit) and update starting prices to 6,600 / 11,200 / 15,400 across site and landing pages
</commit_message>
<xml_diff>
--- a/pricing/OneHome_pricing_model.xlsx
+++ b/pricing/OneHome_pricing_model.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="162">
   <si>
     <t xml:space="preserve">OneHome — מודל תמחור (נבנה מחדש 24/09/2026)</t>
   </si>
@@ -84,10 +84,10 @@
     <t xml:space="preserve">Home Assistant Green: מחיר מומלץ עלה ל-$199 (Nabu Casa, עדכון 24/04/2026, nabucasa.com/news/2026-01-08-green-pricing-change). כמעט כפול מהמחיר המקורי.</t>
   </si>
   <si>
-    <t xml:space="preserve">שאר מחירי החומרה: הערכות של Claude לפי מחירי קמעונאות באירופה/ארה"ב + יבוא ומע"מ בישראל. לא נבדקו מול ספק ישראלי — לאמת לפני הצעת מחיר אמיתית.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">עלויות חשמלאי: הערכות. לאמת מול החשמלאי הקבוע (PRD 1 סעיף G).</t>
+    <t xml:space="preserve">מחירי חומרה: רוב המוצרים אומתו 24/09 מול יבואנים רשמיים בישראל (Ozzi ל-Shelly, Aqara Israel). מה שלא אומת מסומן בקטלוג "הערכה — לא אומת".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">עבודת חשמלאי: 495 ₪ ביקור (PRD 1) + 100 ₪ לכל נקודה נוספת (הערכה). ייחוס: מידרג — התקנת מפסק חכם בודד ≈ 382 ₪ ממוצע (220–495, יולי 2025).</t>
   </si>
   <si>
     <t xml:space="preserve">קטלוג מוצרים ומחיר ללקוח</t>
@@ -138,7 +138,7 @@
     <t xml:space="preserve">בסיס</t>
   </si>
   <si>
-    <t xml:space="preserve">$199 MSRP + יבוא. ההגדרה כלולה בשעות הבסיס.</t>
+    <t xml:space="preserve">נגזר: MSRP $199 (Nabu Casa, 24/04/2026) × 3.7 + מע"מ. לא נמצא מחיר בחנות ישראלית.</t>
   </si>
   <si>
     <t xml:space="preserve">ZBT</t>
@@ -147,7 +147,7 @@
     <t xml:space="preserve">מתאם Zigbee/Thread (Connect ZBT / SkyConnect)</t>
   </si>
   <si>
-    <t xml:space="preserve">ההגדרה כלולה בשעות הבסיס.</t>
+    <t xml:space="preserve">ההגדרה כלולה בשעות הבסיס. · הערכה — לא אומת.</t>
   </si>
   <si>
     <t xml:space="preserve">FP2</t>
@@ -162,7 +162,7 @@
     <t xml:space="preserve">חדר</t>
   </si>
   <si>
-    <t xml:space="preserve">הגדרת אזורים בחדר. דורש מתאם חשמל.</t>
+    <t xml:space="preserve">אומת 24/09 — Aqara Israel, יבואן רשמי (aqaraisrael.co.il), כולל מע"מ. חלופה זולה: FP300 (שורה נפרדת).</t>
   </si>
   <si>
     <t xml:space="preserve">PIR</t>
@@ -171,6 +171,9 @@
     <t xml:space="preserve">Aqara Motion P1 (PIR למעברים)</t>
   </si>
   <si>
+    <t xml:space="preserve">אומת 24/09 — Aqara Israel, יבואן רשמי (aqaraisrael.co.il), כולל מע"מ.</t>
+  </si>
+  <si>
     <t xml:space="preserve">IR</t>
   </si>
   <si>
@@ -180,7 +183,7 @@
     <t xml:space="preserve">Broadlink RM4 mini (שליטה במזגן IR)</t>
   </si>
   <si>
-    <t xml:space="preserve">לימוד קודי IR למזגן.</t>
+    <t xml:space="preserve">לימוד קודי IR למזגן. · הערכה — לא אומת.</t>
   </si>
   <si>
     <t xml:space="preserve">TMP</t>
@@ -189,12 +192,18 @@
     <t xml:space="preserve">חיישן טמפ'/לחות Aqara</t>
   </si>
   <si>
+    <t xml:space="preserve">אומת 24/09 — Aqara Israel, יבואן רשמי (aqaraisrael.co.il), כולל מע"מ. (T1)</t>
+  </si>
+  <si>
     <t xml:space="preserve">AIR</t>
   </si>
   <si>
     <t xml:space="preserve">IKEA VINDSTYRKA (איכות אוויר)</t>
   </si>
   <si>
+    <t xml:space="preserve"> · הערכה — לא אומת.</t>
+  </si>
+  <si>
     <t xml:space="preserve">LEAK</t>
   </si>
   <si>
@@ -204,7 +213,7 @@
     <t xml:space="preserve">חיישן הצפה Aqara</t>
   </si>
   <si>
-    <t xml:space="preserve">אחד כלול בבסיס; נוספים ליד מדיח/מכונת כביסה/דוד.</t>
+    <t xml:space="preserve">אומת 24/09 — Aqara Israel, יבואן רשמי (aqaraisrael.co.il), כולל מע"מ. (T1). אחד כלול בבסיס.</t>
   </si>
   <si>
     <t xml:space="preserve">SMOKE</t>
@@ -213,7 +222,7 @@
     <t xml:space="preserve">גלאי עשן Zigbee</t>
   </si>
   <si>
-    <t xml:space="preserve">אחד כלול בבסיס.</t>
+    <t xml:space="preserve">אומת 24/09 — Aqara Israel, יבואן רשמי (aqaraisrael.co.il), כולל מע"מ. אזל במלאי ביום הבדיקה. אחד כלול בבסיס.</t>
   </si>
   <si>
     <t xml:space="preserve">DIN</t>
@@ -225,7 +234,7 @@
     <t xml:space="preserve">בית</t>
   </si>
   <si>
-    <t xml:space="preserve">עבודת חשמלאי בלוח.</t>
+    <t xml:space="preserve">עבודת חשמלאי בלוח. · הערכה — לא אומת.</t>
   </si>
   <si>
     <t xml:space="preserve">BOIL</t>
@@ -237,25 +246,25 @@
     <t xml:space="preserve">Switcher (בקרת דוד)</t>
   </si>
   <si>
-    <t xml:space="preserve">עבודת חשמלאי.</t>
+    <t xml:space="preserve">עבודת חשמלאי. · הערכה — לא אומת.</t>
   </si>
   <si>
     <t xml:space="preserve">EM1</t>
   </si>
   <si>
-    <t xml:space="preserve">Shelly EM (מדידה חד-פאזית)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">צבת מדידה בלוח — חשמלאי.</t>
+    <t xml:space="preserve">Shelly Pro EM50 (מדידה חד-פאזית)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אומת 24/09 — Ozzi, יבואן Shelly רשמי (ozzi.co.il), כולל מע"מ. (Pro EM50, מדידת בית שלם חד-פאזי).</t>
   </si>
   <si>
     <t xml:space="preserve">EM3</t>
   </si>
   <si>
-    <t xml:space="preserve">Shelly Pro 3EM (מדידה תלת-פאזית)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">חשמלאי.</t>
+    <t xml:space="preserve">Shelly 3EM-63 Gen3 (מדידה תלת-פאזית)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אומת 24/09 — Ozzi, יבואן Shelly רשמי (ozzi.co.il), כולל מע"מ. (3EM-63 Gen3; Pro 3EM 120A = 825 ₪).</t>
   </si>
   <si>
     <t xml:space="preserve">SW1</t>
@@ -264,22 +273,28 @@
     <t xml:space="preserve">6. מפסקים</t>
   </si>
   <si>
-    <t xml:space="preserve">Shelly 1PM (מתג תאורה, לכל נקודה)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">מאחורי מתג קיים — חשמלאי.</t>
+    <t xml:space="preserve">Shelly 1PM Gen4 (מתג תאורה, לכל נקודה)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אומת 24/09 — Ozzi, יבואן Shelly רשמי (ozzi.co.il), כולל מע"מ. (1PM Gen4). חשמלאי: 100 ₪ לנקודה נוספת באותו ביקור — הערכה; מידרג: התקנת מפסק חכם בודד כעבודה נפרדת ≈ 382 ₪ בממוצע (220–495).</t>
   </si>
   <si>
     <t xml:space="preserve">SW2</t>
   </si>
   <si>
-    <t xml:space="preserve">Shelly 2PM (תריס חשמלי)</t>
+    <t xml:space="preserve">Shelly 2PM Gen4 (תריס חשמלי)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אומת 24/09 — Ozzi, יבואן Shelly רשמי (ozzi.co.il), כולל מע"מ. (2PM Gen4, החל מ-159).</t>
   </si>
   <si>
     <t xml:space="preserve">DIM</t>
   </si>
   <si>
-    <t xml:space="preserve">Shelly Dimmer (עמעם)</t>
+    <t xml:space="preserve">Shelly Dimmer Gen4 (עמעם)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אומת 24/09 — Ozzi, יבואן Shelly רשמי (ozzi.co.il), כולל מע"מ. (Dimmer Gen4).</t>
   </si>
   <si>
     <t xml:space="preserve">DOOR</t>
@@ -291,7 +306,7 @@
     <t xml:space="preserve">חיישן פתיחה/סגירה (דלת/חלון)</t>
   </si>
   <si>
-    <t xml:space="preserve">אחד (דלת כניסה) כלול בבסיס.</t>
+    <t xml:space="preserve">אומת 24/09 — Aqara Israel, יבואן רשמי (aqaraisrael.co.il), כולל מע"מ. (T1, אזל במלאי; P2 עם Matter = 109 ₪). אחד כלול בבסיס.</t>
   </si>
   <si>
     <t xml:space="preserve">LOCK</t>
@@ -303,13 +318,16 @@
     <t xml:space="preserve">תוספת</t>
   </si>
   <si>
-    <t xml:space="preserve">לייף-סטייל, תוספת בתשלום.</t>
+    <t xml:space="preserve">לייף-סטייל, תוספת בתשלום. · הערכה — לא אומת.</t>
   </si>
   <si>
     <t xml:space="preserve">BELL</t>
   </si>
   <si>
-    <t xml:space="preserve">פעמון וידאו</t>
+    <t xml:space="preserve">פעמון וידאו Aqara G410</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אומת 24/09 — Aqara Israel, יבואן רשמי (aqaraisrael.co.il), כולל מע"מ. (Doorbell Camera Hub G410).</t>
   </si>
   <si>
     <t xml:space="preserve">LIGHT</t>
@@ -336,7 +354,7 @@
     <t xml:space="preserve">טאבלט קיר + מתקן</t>
   </si>
   <si>
-    <t xml:space="preserve">כולל הגדרת דשבורד קיר.</t>
+    <t xml:space="preserve">כולל הגדרת דשבורד קיר. · הערכה — לא אומת.</t>
   </si>
   <si>
     <t xml:space="preserve">VOICE</t>
@@ -345,7 +363,7 @@
     <t xml:space="preserve">Home Assistant Voice PE (קולי מקומי)</t>
   </si>
   <si>
-    <t xml:space="preserve">$59 MSRP. פייפליין מקומי Whisper/Piper.</t>
+    <t xml:space="preserve">$59 MSRP × שער + מע"מ. פייפליין מקומי Whisper/Piper.</t>
   </si>
   <si>
     <t xml:space="preserve">CAM</t>
@@ -354,7 +372,31 @@
     <t xml:space="preserve">מצלמת IP (PoE)</t>
   </si>
   <si>
-    <t xml:space="preserve">הקלטה מקומית. ללא WebRTC ענני כברירת מחדל.</t>
+    <t xml:space="preserve">הקלטה מקומית. ללא WebRTC ענני כברירת מחדל. · הערכה — לא אומת.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FP300</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aqara FP300 (נוכחות על סוללה, Zigbee/Thread) — חלופה ל-FP2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אומת 24/09 — Aqara Israel, יבואן רשמי (aqaraisrael.co.il), כולל מע"מ. זול ב-150 ₪ מ-FP2 ולא צריך שקע; פחות אזורים.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOIL2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ערכת Shelly לדוד (שליטה + מדידת טמפ' מים) — חלופה ל-Switcher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אומת 24/09 — Ozzi, יבואן Shelly רשמי (ozzi.co.il), כולל מע"מ. (ערכה דור 3).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOCK2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מנעול חכם Aqara U200 — חלופה ל-Nuki</t>
   </si>
   <si>
     <t xml:space="preserve">החבילה הבסיסית (חובה לכל לקוח)</t>
@@ -411,7 +453,7 @@
     <t xml:space="preserve">נקודות התחלה (Eco / Safe / Elite) — כיול מול המחירים מ-16/09</t>
   </si>
   <si>
-    <t xml:space="preserve">כמויות מעבר לחבילה הבסיסית, לבית טיפוסי. משמשות כהצעה מוכנה בבנייה לפי חדרים.</t>
+    <t xml:space="preserve">כמויות מעבר לחבילה הבסיסית, לבית טיפוסי (גרסה רזה 24/09: FP300 במקום FP2, ערכת Shelly לדוד במקום Switcher, בלי מד חשמל ב-Eco). משמשות כהצעה מוכנה בבנייה לפי חדרים.</t>
   </si>
   <si>
     <t xml:space="preserve">EcoHome</t>
@@ -445,6 +487,9 @@
   </si>
   <si>
     <t xml:space="preserve">פער מהיעד (₪)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מחיר מומלץ לפרסום (מעוגל ל-100)</t>
   </si>
   <si>
     <t xml:space="preserve">אם הפער חיובי ומשמעותי, המחירים מ-16/09 לא מכסים את העלויות בהנחות הנוכחיות (בעיקר בגלל עליית מחיר HA Green ועבודת חשמלאי). ההחלטה — להעלות מחיר, לצמצם כמויות בנקודת ההתחלה, או לעדכן הנחות — אצל גיא.</t>
@@ -472,14 +517,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0%"/>
     <numFmt numFmtId="167" formatCode="#,##0.00"/>
     <numFmt numFmtId="168" formatCode="\₪#,##0;&quot;(₪&quot;#,##0\);\-"/>
     <numFmt numFmtId="169" formatCode="#,##0;\(#,##0\);\-"/>
-    <numFmt numFmtId="170" formatCode="General"/>
+    <numFmt numFmtId="170" formatCode="\₪#,##0"/>
+    <numFmt numFmtId="171" formatCode="General"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -636,7 +682,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -741,11 +787,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="170" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1163,7 +1213,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -1327,7 +1377,7 @@
         <v>43</v>
       </c>
       <c r="D7" s="12" t="n">
-        <v>400</v>
+        <v>349</v>
       </c>
       <c r="E7" s="13" t="n">
         <v>30</v>
@@ -1340,7 +1390,7 @@
       </c>
       <c r="H7" s="14" t="n">
         <f aca="false">ROUNDUP((D7*(1+הנחות!$B$6)+E7/60*הנחות!$B$5+F7)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>610</v>
+        <v>550</v>
       </c>
       <c r="I7" s="11" t="s">
         <v>44</v>
@@ -1360,7 +1410,7 @@
         <v>47</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>130</v>
+        <v>89</v>
       </c>
       <c r="E8" s="13" t="n">
         <v>10</v>
@@ -1373,22 +1423,24 @@
       </c>
       <c r="H8" s="14" t="n">
         <f aca="false">ROUNDUP((D8*(1+הנחות!$B$6)+E8/60*הנחות!$B$5+F8)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="I8" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J8" s="11"/>
+      <c r="J8" s="11" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D9" s="12" t="n">
         <v>110</v>
@@ -1410,21 +1462,21 @@
         <v>44</v>
       </c>
       <c r="J9" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="E10" s="13" t="n">
         <v>10</v>
@@ -1437,22 +1489,24 @@
       </c>
       <c r="H10" s="14" t="n">
         <f aca="false">ROUNDUP((D10*(1+הנחות!$B$6)+E10/60*הנחות!$B$5+F10)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="I10" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="11"/>
+      <c r="J10" s="11" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D11" s="12" t="n">
         <v>200</v>
@@ -1473,20 +1527,22 @@
       <c r="I11" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J11" s="11"/>
+      <c r="J11" s="11" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D12" s="12" t="n">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="E12" s="13" t="n">
         <v>10</v>
@@ -1499,27 +1555,27 @@
       </c>
       <c r="H12" s="14" t="n">
         <f aca="false">ROUNDUP((D12*(1+הנחות!$B$6)+E12/60*הנחות!$B$5+F12)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="I12" s="11" t="s">
         <v>44</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>57</v>
-      </c>
       <c r="C13" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D13" s="12" t="n">
-        <v>200</v>
+        <v>159</v>
       </c>
       <c r="E13" s="13" t="n">
         <v>15</v>
@@ -1532,24 +1588,24 @@
       </c>
       <c r="H13" s="14" t="n">
         <f aca="false">ROUNDUP((D13*(1+הנחות!$B$6)+E13/60*הנחות!$B$5+F13)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>310</v>
+        <v>260</v>
       </c>
       <c r="I13" s="11" t="s">
         <v>44</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D14" s="12" t="n">
         <v>350</v>
@@ -1568,21 +1624,21 @@
         <v>820</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D15" s="12" t="n">
         <v>380</v>
@@ -1601,24 +1657,24 @@
         <v>810</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>68</v>
-      </c>
       <c r="C16" s="11" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D16" s="12" t="n">
-        <v>300</v>
+        <v>529</v>
       </c>
       <c r="E16" s="13" t="n">
         <v>15</v>
@@ -1631,27 +1687,27 @@
       </c>
       <c r="H16" s="14" t="n">
         <f aca="false">ROUNDUP((D16*(1+הנחות!$B$6)+E16/60*הנחות!$B$5+F16)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>690</v>
+        <v>990</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D17" s="12" t="n">
-        <v>650</v>
+        <v>495</v>
       </c>
       <c r="E17" s="13" t="n">
         <v>20</v>
@@ -1664,99 +1720,99 @@
       </c>
       <c r="H17" s="14" t="n">
         <f aca="false">ROUNDUP((D17*(1+הנחות!$B$6)+E17/60*הנחות!$B$5+F17)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>1260</v>
+        <v>1060</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D18" s="12" t="n">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="E18" s="13" t="n">
         <v>10</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>1</v>
       </c>
       <c r="H18" s="14" t="n">
         <f aca="false">ROUNDUP((D18*(1+הנחות!$B$6)+E18/60*הנחות!$B$5+F18)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>330</v>
+        <v>280</v>
       </c>
       <c r="I18" s="11" t="s">
         <v>44</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B19" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="B19" s="11" t="s">
-        <v>78</v>
-      </c>
       <c r="C19" s="11" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D19" s="12" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E19" s="13" t="n">
         <v>15</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G19" s="13" t="n">
         <v>1</v>
       </c>
       <c r="H19" s="14" t="n">
         <f aca="false">ROUNDUP((D19*(1+הנחות!$B$6)+E19/60*הנחות!$B$5+F19)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>410</v>
+        <v>360</v>
       </c>
       <c r="I19" s="11" t="s">
         <v>44</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D20" s="12" t="n">
-        <v>170</v>
+        <v>212</v>
       </c>
       <c r="E20" s="13" t="n">
         <v>10</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G20" s="13" t="n">
         <v>1</v>
@@ -1769,21 +1825,21 @@
         <v>44</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D21" s="12" t="n">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E21" s="13" t="n">
         <v>10</v>
@@ -1796,24 +1852,24 @@
       </c>
       <c r="H21" s="14" t="n">
         <f aca="false">ROUNDUP((D21*(1+הנחות!$B$6)+E21/60*הנחות!$B$5+F21)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="I21" s="11" t="s">
         <v>44</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D22" s="12" t="n">
         <v>1200</v>
@@ -1832,24 +1888,24 @@
         <v>1700</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D23" s="12" t="n">
-        <v>550</v>
+        <v>599</v>
       </c>
       <c r="E23" s="13" t="n">
         <v>45</v>
@@ -1862,24 +1918,24 @@
       </c>
       <c r="H23" s="14" t="n">
         <f aca="false">ROUNDUP((D23*(1+הנחות!$B$6)+E23/60*הנחות!$B$5+F23)/הנחות!$B$10,0)*הנחות!$B$10</f>
-        <v>850</v>
+        <v>920</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="D24" s="12" t="n">
         <v>120</v>
@@ -1898,19 +1954,21 @@
         <v>190</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="J24" s="11"/>
+        <v>96</v>
+      </c>
+      <c r="J24" s="11" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D25" s="12" t="n">
         <v>70</v>
@@ -1929,19 +1987,21 @@
         <v>130</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="J25" s="11"/>
+        <v>96</v>
+      </c>
+      <c r="J25" s="11" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D26" s="12" t="n">
         <v>900</v>
@@ -1960,21 +2020,21 @@
         <v>1440</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="D27" s="12" t="n">
         <v>330</v>
@@ -1993,21 +2053,21 @@
         <v>570</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D28" s="12" t="n">
         <v>400</v>
@@ -2026,10 +2086,109 @@
         <v>610</v>
       </c>
       <c r="I28" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="J28" s="11" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>199</v>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="14" t="n">
+        <f aca="false">ROUNDUP((D29*(1+הנחות!$B$6)+E29/60*הנחות!$B$5+F29)/הנחות!$B$10,0)*הנחות!$B$10</f>
+        <v>320</v>
+      </c>
+      <c r="I29" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="J29" s="11" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D30" s="12" t="n">
+        <v>189</v>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="F30" s="12" t="n">
+        <v>250</v>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="14" t="n">
+        <f aca="false">ROUNDUP((D30*(1+הנחות!$B$6)+E30/60*הנחות!$B$5+F30)/הנחות!$B$10,0)*הנחות!$B$10</f>
+        <v>560</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="J30" s="11" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B31" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="J28" s="11" t="s">
-        <v>109</v>
+      <c r="C31" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="D31" s="12" t="n">
+        <v>899</v>
+      </c>
+      <c r="E31" s="13" t="n">
+        <v>45</v>
+      </c>
+      <c r="F31" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="14" t="n">
+        <f aca="false">ROUNDUP((D31*(1+הנחות!$B$6)+E31/60*הנחות!$B$5+F31)/הנחות!$B$10,0)*הנחות!$B$10</f>
+        <v>1310</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="J31" s="11" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2060,7 +2219,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2076,19 +2235,19 @@
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2143,11 +2302,11 @@
       </c>
       <c r="C6" s="17" t="n">
         <f aca="false">קטלוג!H12</f>
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="D6" s="18" t="n">
         <f aca="false">B6*C6</f>
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="E6" s="3" t="n">
         <f aca="false">B6*קטלוג!G12</f>
@@ -2164,11 +2323,11 @@
       </c>
       <c r="C7" s="17" t="n">
         <f aca="false">קטלוג!H13</f>
-        <v>310</v>
+        <v>260</v>
       </c>
       <c r="D7" s="18" t="n">
         <f aca="false">B7*C7</f>
-        <v>310</v>
+        <v>260</v>
       </c>
       <c r="E7" s="3" t="n">
         <f aca="false">B7*קטלוג!G13</f>
@@ -2185,11 +2344,11 @@
       </c>
       <c r="C8" s="17" t="n">
         <f aca="false">קטלוג!H21</f>
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D8" s="18" t="n">
         <f aca="false">B8*C8</f>
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="E8" s="3" t="n">
         <f aca="false">B8*קטלוג!G21</f>
@@ -2198,7 +2357,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="B9" s="19" t="n">
         <f aca="false">הנחות!$B$8</f>
@@ -2216,13 +2375,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="20" t="n">
         <f aca="false">SUM(D4:D9)</f>
-        <v>3170</v>
+        <v>3100</v>
       </c>
       <c r="E10" s="10" t="n">
         <f aca="false">SUM(E4:E8)</f>
@@ -2255,7 +2414,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2269,13 +2428,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>32</v>
@@ -2292,7 +2451,7 @@
         <v>160</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2306,7 +2465,7 @@
         <v>220</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2314,13 +2473,13 @@
         <v>51</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="C6" s="21" t="n">
         <v>350</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2331,7 +2490,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -2365,7 +2524,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2376,7 +2535,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2399,48 +2558,48 @@
         <v>25</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="G4" s="22" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="str">
-        <f aca="false">קטלוג!C7</f>
-        <v>Aqara FP2 (חיישן נוכחות mmWave)</v>
+        <f aca="false">קטלוג!C29</f>
+        <v>Aqara FP300 (נוכחות על סוללה, Zigbee/Thread) — חלופה ל-FP2</v>
       </c>
       <c r="B5" s="17" t="n">
-        <f aca="false">קטלוג!H7</f>
-        <v>610</v>
+        <f aca="false">קטלוג!H29</f>
+        <v>320</v>
       </c>
       <c r="C5" s="16" t="n">
         <v>2</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F5" s="17" t="n">
-        <f aca="false">קטלוג!F7</f>
+        <f aca="false">קטלוג!F29</f>
         <v>0</v>
       </c>
       <c r="G5" s="15" t="n">
-        <f aca="false">קטלוג!G7</f>
+        <f aca="false">קטלוג!G29</f>
         <v>1</v>
       </c>
     </row>
@@ -2451,7 +2610,7 @@
       </c>
       <c r="B6" s="17" t="n">
         <f aca="false">קטלוג!H8</f>
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C6" s="16" t="n">
         <v>1</v>
@@ -2460,7 +2619,7 @@
         <v>2</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" s="17" t="n">
         <f aca="false">קטלוג!F8</f>
@@ -2505,7 +2664,7 @@
       </c>
       <c r="B8" s="17" t="n">
         <f aca="false">קטלוג!H10</f>
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="C8" s="16" t="n">
         <v>1</v>
@@ -2559,7 +2718,7 @@
       </c>
       <c r="B10" s="17" t="n">
         <f aca="false">קטלוג!H12</f>
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="C10" s="16" t="n">
         <v>0</v>
@@ -2608,12 +2767,12 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="str">
-        <f aca="false">קטלוג!C15</f>
-        <v>Switcher (בקרת דוד)</v>
+        <f aca="false">קטלוג!C30</f>
+        <v>ערכת Shelly לדוד (שליטה + מדידת טמפ' מים) — חלופה ל-Switcher</v>
       </c>
       <c r="B12" s="17" t="n">
-        <f aca="false">קטלוג!H15</f>
-        <v>810</v>
+        <f aca="false">קטלוג!H30</f>
+        <v>560</v>
       </c>
       <c r="C12" s="16" t="n">
         <v>1</v>
@@ -2625,25 +2784,25 @@
         <v>1</v>
       </c>
       <c r="F12" s="17" t="n">
-        <f aca="false">קטלוג!F15</f>
+        <f aca="false">קטלוג!F30</f>
         <v>250</v>
       </c>
       <c r="G12" s="15" t="n">
-        <f aca="false">קטלוג!G15</f>
+        <f aca="false">קטלוג!G30</f>
         <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="str">
         <f aca="false">קטלוג!C16</f>
-        <v>Shelly EM (מדידה חד-פאזית)</v>
+        <v>Shelly Pro EM50 (מדידה חד-פאזית)</v>
       </c>
       <c r="B13" s="17" t="n">
         <f aca="false">קטלוג!H16</f>
-        <v>690</v>
+        <v>990</v>
       </c>
       <c r="C13" s="16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" s="16" t="n">
         <v>1</v>
@@ -2663,11 +2822,11 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="str">
         <f aca="false">קטלוג!C17</f>
-        <v>Shelly Pro 3EM (מדידה תלת-פאזית)</v>
+        <v>Shelly 3EM-63 Gen3 (מדידה תלת-פאזית)</v>
       </c>
       <c r="B14" s="17" t="n">
         <f aca="false">קטלוג!H17</f>
-        <v>1260</v>
+        <v>1060</v>
       </c>
       <c r="C14" s="16" t="n">
         <v>0</v>
@@ -2690,11 +2849,11 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="str">
         <f aca="false">קטלוג!C18</f>
-        <v>Shelly 1PM (מתג תאורה, לכל נקודה)</v>
+        <v>Shelly 1PM Gen4 (מתג תאורה, לכל נקודה)</v>
       </c>
       <c r="B15" s="17" t="n">
         <f aca="false">קטלוג!H18</f>
-        <v>330</v>
+        <v>280</v>
       </c>
       <c r="C15" s="16" t="n">
         <v>3</v>
@@ -2703,11 +2862,11 @@
         <v>5</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F15" s="17" t="n">
         <f aca="false">קטלוג!F18</f>
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G15" s="15" t="n">
         <f aca="false">קטלוג!G18</f>
@@ -2717,11 +2876,11 @@
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="str">
         <f aca="false">קטלוג!C19</f>
-        <v>Shelly 2PM (תריס חשמלי)</v>
+        <v>Shelly 2PM Gen4 (תריס חשמלי)</v>
       </c>
       <c r="B16" s="17" t="n">
         <f aca="false">קטלוג!H19</f>
-        <v>410</v>
+        <v>360</v>
       </c>
       <c r="C16" s="16" t="n">
         <v>0</v>
@@ -2730,11 +2889,11 @@
         <v>2</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F16" s="17" t="n">
         <f aca="false">קטלוג!F19</f>
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G16" s="15" t="n">
         <f aca="false">קטלוג!G19</f>
@@ -2744,7 +2903,7 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="str">
         <f aca="false">קטלוג!C20</f>
-        <v>Shelly Dimmer (עמעם)</v>
+        <v>Shelly Dimmer Gen4 (עמעם)</v>
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">קטלוג!H20</f>
@@ -2754,14 +2913,14 @@
         <v>0</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17" s="17" t="n">
         <f aca="false">קטלוג!F20</f>
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G17" s="15" t="n">
         <f aca="false">קטלוג!G20</f>
@@ -2775,16 +2934,16 @@
       </c>
       <c r="B18" s="17" t="n">
         <f aca="false">קטלוג!H21</f>
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C18" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E18" s="16" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F18" s="17" t="n">
         <f aca="false">קטלוג!F21</f>
@@ -2806,47 +2965,47 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="23" t="n">
         <f aca="false">SUMPRODUCT($B$5:$B$18,C5:C18)</f>
-        <v>4820</v>
+        <v>2930</v>
       </c>
       <c r="D20" s="23" t="n">
         <f aca="false">SUMPRODUCT($B$5:$B$18,D5:D18)</f>
-        <v>10210</v>
+        <v>7590</v>
       </c>
       <c r="E20" s="23" t="n">
         <f aca="false">SUMPRODUCT($B$5:$B$18,E5:E18)</f>
-        <v>17290</v>
+        <v>11710</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="23" t="n">
         <f aca="false">'חבילה בסיסית'!$D$10</f>
-        <v>3170</v>
+        <v>3100</v>
       </c>
       <c r="D21" s="23" t="n">
         <f aca="false">'חבילה בסיסית'!$D$10</f>
-        <v>3170</v>
+        <v>3100</v>
       </c>
       <c r="E21" s="23" t="n">
         <f aca="false">'חבילה בסיסית'!$D$10</f>
-        <v>3170</v>
+        <v>3100</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="23" t="n">
@@ -2866,27 +3025,27 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="20" t="n">
         <f aca="false">SUM(C20:C22)</f>
-        <v>8485</v>
+        <v>6525</v>
       </c>
       <c r="D23" s="20" t="n">
         <f aca="false">SUM(D20:D22)</f>
-        <v>13875</v>
+        <v>11185</v>
       </c>
       <c r="E23" s="20" t="n">
         <f aca="false">SUM(E20:E22)</f>
-        <v>20955</v>
+        <v>15305</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="24" t="n">
@@ -2903,47 +3062,47 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="23" t="n">
         <f aca="false">C23-C24</f>
-        <v>2785</v>
+        <v>825</v>
       </c>
       <c r="D25" s="23" t="n">
         <f aca="false">D23-D24</f>
-        <v>5175</v>
+        <v>2485</v>
       </c>
       <c r="E25" s="23" t="n">
         <f aca="false">E23-E24</f>
-        <v>7805</v>
+        <v>2155</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="25" t="n">
         <f aca="false">'חבילה בסיסית'!$E$10+SUMPRODUCT($G$5:$G$18,C5:C18)</f>
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D26" s="25" t="n">
         <f aca="false">'חבילה בסיסית'!$E$10+SUMPRODUCT($G$5:$G$18,D5:D18)</f>
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E26" s="25" t="n">
         <f aca="false">'חבילה בסיסית'!$E$10+SUMPRODUCT($G$5:$G$18,E5:E18)</f>
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="23" t="n">
@@ -2956,23 +3115,34 @@
       </c>
       <c r="E27" s="23" t="n">
         <f aca="false">INDEX(ריטיינר!$C$4:$C$6,MATCH(E26,ריטיינר!$A$4:$A$6,1))</f>
-        <v>350</v>
+        <v>220</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3"/>
+      <c r="A28" s="10" t="s">
+        <v>154</v>
+      </c>
       <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
+      <c r="C28" s="26" t="n">
+        <f aca="false">ROUNDUP(C23/100,0)*100</f>
+        <v>6600</v>
+      </c>
+      <c r="D28" s="26" t="n">
+        <f aca="false">ROUNDUP(D23/100,0)*100</f>
+        <v>11200</v>
+      </c>
+      <c r="E28" s="26" t="n">
+        <f aca="false">ROUNDUP(E23/100,0)*100</f>
+        <v>15400</v>
+      </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -3011,7 +3181,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3022,7 +3192,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3048,45 +3218,45 @@
         <v>25</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="26" t="n">
-        <f aca="false">IF(B5="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B5,קטלוג!$C$5:$C$28,0)))</f>
-        <v>330</v>
-      </c>
-      <c r="E5" s="26" t="n">
+      <c r="D5" s="27" t="n">
+        <f aca="false">IF(B5="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B5,קטלוג!$C$5:$C$31,0)))</f>
+        <v>280</v>
+      </c>
+      <c r="E5" s="27" t="n">
         <f aca="false">IF(B5="","",C5*D5)</f>
-        <v>990</v>
-      </c>
-      <c r="F5" s="27" t="n">
-        <f aca="false">IF(B5="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B5,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v>1</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <f aca="false">IF(B5="","",C5*INDEX(קטלוג!$G$5:$G$28,MATCH(B5,קטלוג!$C$5:$C$28,0)))</f>
+        <v>840</v>
+      </c>
+      <c r="F5" s="28" t="n">
+        <f aca="false">IF(B5="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B5,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v>1</v>
+      </c>
+      <c r="G5" s="28" t="n">
+        <f aca="false">IF(B5="","",C5*INDEX(קטלוג!$G$5:$G$31,MATCH(B5,קטלוג!$C$5:$C$31,0)))</f>
         <v>3</v>
       </c>
     </row>
@@ -3094,20 +3264,20 @@
       <c r="A6" s="13"/>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
-      <c r="D6" s="26" t="str">
-        <f aca="false">IF(B6="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B6,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E6" s="26" t="str">
+      <c r="D6" s="27" t="str">
+        <f aca="false">IF(B6="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B6,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E6" s="27" t="str">
         <f aca="false">IF(B6="","",C6*D6)</f>
         <v/>
       </c>
-      <c r="F6" s="27" t="str">
-        <f aca="false">IF(B6="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B6,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G6" s="27" t="str">
-        <f aca="false">IF(B6="","",C6*INDEX(קטלוג!$G$5:$G$28,MATCH(B6,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F6" s="28" t="str">
+        <f aca="false">IF(B6="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B6,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G6" s="28" t="str">
+        <f aca="false">IF(B6="","",C6*INDEX(קטלוג!$G$5:$G$31,MATCH(B6,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3115,20 +3285,20 @@
       <c r="A7" s="13"/>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
-      <c r="D7" s="26" t="str">
-        <f aca="false">IF(B7="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B7,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E7" s="26" t="str">
+      <c r="D7" s="27" t="str">
+        <f aca="false">IF(B7="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B7,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E7" s="27" t="str">
         <f aca="false">IF(B7="","",C7*D7)</f>
         <v/>
       </c>
-      <c r="F7" s="27" t="str">
-        <f aca="false">IF(B7="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B7,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G7" s="27" t="str">
-        <f aca="false">IF(B7="","",C7*INDEX(קטלוג!$G$5:$G$28,MATCH(B7,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F7" s="28" t="str">
+        <f aca="false">IF(B7="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B7,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G7" s="28" t="str">
+        <f aca="false">IF(B7="","",C7*INDEX(קטלוג!$G$5:$G$31,MATCH(B7,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3136,20 +3306,20 @@
       <c r="A8" s="13"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
-      <c r="D8" s="26" t="str">
-        <f aca="false">IF(B8="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B8,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E8" s="26" t="str">
+      <c r="D8" s="27" t="str">
+        <f aca="false">IF(B8="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B8,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E8" s="27" t="str">
         <f aca="false">IF(B8="","",C8*D8)</f>
         <v/>
       </c>
-      <c r="F8" s="27" t="str">
-        <f aca="false">IF(B8="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B8,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G8" s="27" t="str">
-        <f aca="false">IF(B8="","",C8*INDEX(קטלוג!$G$5:$G$28,MATCH(B8,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F8" s="28" t="str">
+        <f aca="false">IF(B8="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B8,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G8" s="28" t="str">
+        <f aca="false">IF(B8="","",C8*INDEX(קטלוג!$G$5:$G$31,MATCH(B8,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3157,20 +3327,20 @@
       <c r="A9" s="13"/>
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
-      <c r="D9" s="26" t="str">
-        <f aca="false">IF(B9="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B9,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E9" s="26" t="str">
+      <c r="D9" s="27" t="str">
+        <f aca="false">IF(B9="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B9,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E9" s="27" t="str">
         <f aca="false">IF(B9="","",C9*D9)</f>
         <v/>
       </c>
-      <c r="F9" s="27" t="str">
-        <f aca="false">IF(B9="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B9,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G9" s="27" t="str">
-        <f aca="false">IF(B9="","",C9*INDEX(קטלוג!$G$5:$G$28,MATCH(B9,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F9" s="28" t="str">
+        <f aca="false">IF(B9="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B9,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G9" s="28" t="str">
+        <f aca="false">IF(B9="","",C9*INDEX(קטלוג!$G$5:$G$31,MATCH(B9,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3178,20 +3348,20 @@
       <c r="A10" s="13"/>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
-      <c r="D10" s="26" t="str">
-        <f aca="false">IF(B10="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B10,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E10" s="26" t="str">
+      <c r="D10" s="27" t="str">
+        <f aca="false">IF(B10="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B10,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E10" s="27" t="str">
         <f aca="false">IF(B10="","",C10*D10)</f>
         <v/>
       </c>
-      <c r="F10" s="27" t="str">
-        <f aca="false">IF(B10="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B10,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G10" s="27" t="str">
-        <f aca="false">IF(B10="","",C10*INDEX(קטלוג!$G$5:$G$28,MATCH(B10,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F10" s="28" t="str">
+        <f aca="false">IF(B10="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B10,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G10" s="28" t="str">
+        <f aca="false">IF(B10="","",C10*INDEX(קטלוג!$G$5:$G$31,MATCH(B10,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3199,20 +3369,20 @@
       <c r="A11" s="13"/>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
-      <c r="D11" s="26" t="str">
-        <f aca="false">IF(B11="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B11,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E11" s="26" t="str">
+      <c r="D11" s="27" t="str">
+        <f aca="false">IF(B11="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B11,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E11" s="27" t="str">
         <f aca="false">IF(B11="","",C11*D11)</f>
         <v/>
       </c>
-      <c r="F11" s="27" t="str">
-        <f aca="false">IF(B11="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B11,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G11" s="27" t="str">
-        <f aca="false">IF(B11="","",C11*INDEX(קטלוג!$G$5:$G$28,MATCH(B11,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F11" s="28" t="str">
+        <f aca="false">IF(B11="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B11,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G11" s="28" t="str">
+        <f aca="false">IF(B11="","",C11*INDEX(קטלוג!$G$5:$G$31,MATCH(B11,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3220,20 +3390,20 @@
       <c r="A12" s="13"/>
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
-      <c r="D12" s="26" t="str">
-        <f aca="false">IF(B12="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B12,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E12" s="26" t="str">
+      <c r="D12" s="27" t="str">
+        <f aca="false">IF(B12="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B12,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E12" s="27" t="str">
         <f aca="false">IF(B12="","",C12*D12)</f>
         <v/>
       </c>
-      <c r="F12" s="27" t="str">
-        <f aca="false">IF(B12="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B12,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G12" s="27" t="str">
-        <f aca="false">IF(B12="","",C12*INDEX(קטלוג!$G$5:$G$28,MATCH(B12,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F12" s="28" t="str">
+        <f aca="false">IF(B12="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B12,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G12" s="28" t="str">
+        <f aca="false">IF(B12="","",C12*INDEX(קטלוג!$G$5:$G$31,MATCH(B12,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3241,20 +3411,20 @@
       <c r="A13" s="13"/>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
-      <c r="D13" s="26" t="str">
-        <f aca="false">IF(B13="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B13,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E13" s="26" t="str">
+      <c r="D13" s="27" t="str">
+        <f aca="false">IF(B13="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B13,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E13" s="27" t="str">
         <f aca="false">IF(B13="","",C13*D13)</f>
         <v/>
       </c>
-      <c r="F13" s="27" t="str">
-        <f aca="false">IF(B13="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B13,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G13" s="27" t="str">
-        <f aca="false">IF(B13="","",C13*INDEX(קטלוג!$G$5:$G$28,MATCH(B13,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F13" s="28" t="str">
+        <f aca="false">IF(B13="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B13,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G13" s="28" t="str">
+        <f aca="false">IF(B13="","",C13*INDEX(קטלוג!$G$5:$G$31,MATCH(B13,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3262,20 +3432,20 @@
       <c r="A14" s="13"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
-      <c r="D14" s="26" t="str">
-        <f aca="false">IF(B14="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B14,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E14" s="26" t="str">
+      <c r="D14" s="27" t="str">
+        <f aca="false">IF(B14="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B14,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E14" s="27" t="str">
         <f aca="false">IF(B14="","",C14*D14)</f>
         <v/>
       </c>
-      <c r="F14" s="27" t="str">
-        <f aca="false">IF(B14="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B14,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G14" s="27" t="str">
-        <f aca="false">IF(B14="","",C14*INDEX(קטלוג!$G$5:$G$28,MATCH(B14,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F14" s="28" t="str">
+        <f aca="false">IF(B14="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B14,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G14" s="28" t="str">
+        <f aca="false">IF(B14="","",C14*INDEX(קטלוג!$G$5:$G$31,MATCH(B14,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3283,20 +3453,20 @@
       <c r="A15" s="13"/>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
-      <c r="D15" s="26" t="str">
-        <f aca="false">IF(B15="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B15,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E15" s="26" t="str">
+      <c r="D15" s="27" t="str">
+        <f aca="false">IF(B15="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B15,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E15" s="27" t="str">
         <f aca="false">IF(B15="","",C15*D15)</f>
         <v/>
       </c>
-      <c r="F15" s="27" t="str">
-        <f aca="false">IF(B15="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B15,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G15" s="27" t="str">
-        <f aca="false">IF(B15="","",C15*INDEX(קטלוג!$G$5:$G$28,MATCH(B15,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F15" s="28" t="str">
+        <f aca="false">IF(B15="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B15,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G15" s="28" t="str">
+        <f aca="false">IF(B15="","",C15*INDEX(קטלוג!$G$5:$G$31,MATCH(B15,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3304,20 +3474,20 @@
       <c r="A16" s="13"/>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
-      <c r="D16" s="26" t="str">
-        <f aca="false">IF(B16="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B16,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E16" s="26" t="str">
+      <c r="D16" s="27" t="str">
+        <f aca="false">IF(B16="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B16,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E16" s="27" t="str">
         <f aca="false">IF(B16="","",C16*D16)</f>
         <v/>
       </c>
-      <c r="F16" s="27" t="str">
-        <f aca="false">IF(B16="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B16,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G16" s="27" t="str">
-        <f aca="false">IF(B16="","",C16*INDEX(קטלוג!$G$5:$G$28,MATCH(B16,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F16" s="28" t="str">
+        <f aca="false">IF(B16="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B16,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G16" s="28" t="str">
+        <f aca="false">IF(B16="","",C16*INDEX(קטלוג!$G$5:$G$31,MATCH(B16,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3325,20 +3495,20 @@
       <c r="A17" s="13"/>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
-      <c r="D17" s="26" t="str">
-        <f aca="false">IF(B17="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B17,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E17" s="26" t="str">
+      <c r="D17" s="27" t="str">
+        <f aca="false">IF(B17="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B17,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E17" s="27" t="str">
         <f aca="false">IF(B17="","",C17*D17)</f>
         <v/>
       </c>
-      <c r="F17" s="27" t="str">
-        <f aca="false">IF(B17="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B17,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G17" s="27" t="str">
-        <f aca="false">IF(B17="","",C17*INDEX(קטלוג!$G$5:$G$28,MATCH(B17,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F17" s="28" t="str">
+        <f aca="false">IF(B17="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B17,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G17" s="28" t="str">
+        <f aca="false">IF(B17="","",C17*INDEX(קטלוג!$G$5:$G$31,MATCH(B17,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3346,20 +3516,20 @@
       <c r="A18" s="13"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
-      <c r="D18" s="26" t="str">
-        <f aca="false">IF(B18="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B18,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E18" s="26" t="str">
+      <c r="D18" s="27" t="str">
+        <f aca="false">IF(B18="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B18,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E18" s="27" t="str">
         <f aca="false">IF(B18="","",C18*D18)</f>
         <v/>
       </c>
-      <c r="F18" s="27" t="str">
-        <f aca="false">IF(B18="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B18,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G18" s="27" t="str">
-        <f aca="false">IF(B18="","",C18*INDEX(קטלוג!$G$5:$G$28,MATCH(B18,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F18" s="28" t="str">
+        <f aca="false">IF(B18="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B18,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G18" s="28" t="str">
+        <f aca="false">IF(B18="","",C18*INDEX(קטלוג!$G$5:$G$31,MATCH(B18,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3367,20 +3537,20 @@
       <c r="A19" s="13"/>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
-      <c r="D19" s="26" t="str">
-        <f aca="false">IF(B19="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B19,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E19" s="26" t="str">
+      <c r="D19" s="27" t="str">
+        <f aca="false">IF(B19="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B19,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E19" s="27" t="str">
         <f aca="false">IF(B19="","",C19*D19)</f>
         <v/>
       </c>
-      <c r="F19" s="27" t="str">
-        <f aca="false">IF(B19="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B19,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G19" s="27" t="str">
-        <f aca="false">IF(B19="","",C19*INDEX(קטלוג!$G$5:$G$28,MATCH(B19,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F19" s="28" t="str">
+        <f aca="false">IF(B19="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B19,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G19" s="28" t="str">
+        <f aca="false">IF(B19="","",C19*INDEX(קטלוג!$G$5:$G$31,MATCH(B19,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3388,20 +3558,20 @@
       <c r="A20" s="13"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
-      <c r="D20" s="26" t="str">
-        <f aca="false">IF(B20="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B20,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E20" s="26" t="str">
+      <c r="D20" s="27" t="str">
+        <f aca="false">IF(B20="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B20,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E20" s="27" t="str">
         <f aca="false">IF(B20="","",C20*D20)</f>
         <v/>
       </c>
-      <c r="F20" s="27" t="str">
-        <f aca="false">IF(B20="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B20,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G20" s="27" t="str">
-        <f aca="false">IF(B20="","",C20*INDEX(קטלוג!$G$5:$G$28,MATCH(B20,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F20" s="28" t="str">
+        <f aca="false">IF(B20="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B20,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G20" s="28" t="str">
+        <f aca="false">IF(B20="","",C20*INDEX(קטלוג!$G$5:$G$31,MATCH(B20,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3409,20 +3579,20 @@
       <c r="A21" s="13"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
-      <c r="D21" s="26" t="str">
-        <f aca="false">IF(B21="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B21,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E21" s="26" t="str">
+      <c r="D21" s="27" t="str">
+        <f aca="false">IF(B21="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B21,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E21" s="27" t="str">
         <f aca="false">IF(B21="","",C21*D21)</f>
         <v/>
       </c>
-      <c r="F21" s="27" t="str">
-        <f aca="false">IF(B21="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B21,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G21" s="27" t="str">
-        <f aca="false">IF(B21="","",C21*INDEX(קטלוג!$G$5:$G$28,MATCH(B21,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F21" s="28" t="str">
+        <f aca="false">IF(B21="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B21,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G21" s="28" t="str">
+        <f aca="false">IF(B21="","",C21*INDEX(קטלוג!$G$5:$G$31,MATCH(B21,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3430,20 +3600,20 @@
       <c r="A22" s="13"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
-      <c r="D22" s="26" t="str">
-        <f aca="false">IF(B22="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B22,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E22" s="26" t="str">
+      <c r="D22" s="27" t="str">
+        <f aca="false">IF(B22="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B22,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E22" s="27" t="str">
         <f aca="false">IF(B22="","",C22*D22)</f>
         <v/>
       </c>
-      <c r="F22" s="27" t="str">
-        <f aca="false">IF(B22="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B22,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G22" s="27" t="str">
-        <f aca="false">IF(B22="","",C22*INDEX(קטלוג!$G$5:$G$28,MATCH(B22,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F22" s="28" t="str">
+        <f aca="false">IF(B22="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B22,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G22" s="28" t="str">
+        <f aca="false">IF(B22="","",C22*INDEX(קטלוג!$G$5:$G$31,MATCH(B22,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3451,20 +3621,20 @@
       <c r="A23" s="13"/>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
-      <c r="D23" s="26" t="str">
-        <f aca="false">IF(B23="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B23,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E23" s="26" t="str">
+      <c r="D23" s="27" t="str">
+        <f aca="false">IF(B23="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B23,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E23" s="27" t="str">
         <f aca="false">IF(B23="","",C23*D23)</f>
         <v/>
       </c>
-      <c r="F23" s="27" t="str">
-        <f aca="false">IF(B23="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B23,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G23" s="27" t="str">
-        <f aca="false">IF(B23="","",C23*INDEX(קטלוג!$G$5:$G$28,MATCH(B23,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F23" s="28" t="str">
+        <f aca="false">IF(B23="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B23,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G23" s="28" t="str">
+        <f aca="false">IF(B23="","",C23*INDEX(קטלוג!$G$5:$G$31,MATCH(B23,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3472,20 +3642,20 @@
       <c r="A24" s="13"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
-      <c r="D24" s="26" t="str">
-        <f aca="false">IF(B24="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B24,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E24" s="26" t="str">
+      <c r="D24" s="27" t="str">
+        <f aca="false">IF(B24="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B24,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E24" s="27" t="str">
         <f aca="false">IF(B24="","",C24*D24)</f>
         <v/>
       </c>
-      <c r="F24" s="27" t="str">
-        <f aca="false">IF(B24="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B24,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G24" s="27" t="str">
-        <f aca="false">IF(B24="","",C24*INDEX(קטלוג!$G$5:$G$28,MATCH(B24,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F24" s="28" t="str">
+        <f aca="false">IF(B24="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B24,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G24" s="28" t="str">
+        <f aca="false">IF(B24="","",C24*INDEX(קטלוג!$G$5:$G$31,MATCH(B24,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3493,20 +3663,20 @@
       <c r="A25" s="13"/>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
-      <c r="D25" s="26" t="str">
-        <f aca="false">IF(B25="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B25,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E25" s="26" t="str">
+      <c r="D25" s="27" t="str">
+        <f aca="false">IF(B25="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B25,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E25" s="27" t="str">
         <f aca="false">IF(B25="","",C25*D25)</f>
         <v/>
       </c>
-      <c r="F25" s="27" t="str">
-        <f aca="false">IF(B25="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B25,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G25" s="27" t="str">
-        <f aca="false">IF(B25="","",C25*INDEX(קטלוג!$G$5:$G$28,MATCH(B25,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F25" s="28" t="str">
+        <f aca="false">IF(B25="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B25,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G25" s="28" t="str">
+        <f aca="false">IF(B25="","",C25*INDEX(קטלוג!$G$5:$G$31,MATCH(B25,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3514,20 +3684,20 @@
       <c r="A26" s="13"/>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
-      <c r="D26" s="26" t="str">
-        <f aca="false">IF(B26="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B26,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E26" s="26" t="str">
+      <c r="D26" s="27" t="str">
+        <f aca="false">IF(B26="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B26,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E26" s="27" t="str">
         <f aca="false">IF(B26="","",C26*D26)</f>
         <v/>
       </c>
-      <c r="F26" s="27" t="str">
-        <f aca="false">IF(B26="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B26,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G26" s="27" t="str">
-        <f aca="false">IF(B26="","",C26*INDEX(קטלוג!$G$5:$G$28,MATCH(B26,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F26" s="28" t="str">
+        <f aca="false">IF(B26="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B26,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G26" s="28" t="str">
+        <f aca="false">IF(B26="","",C26*INDEX(קטלוג!$G$5:$G$31,MATCH(B26,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3535,20 +3705,20 @@
       <c r="A27" s="13"/>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
-      <c r="D27" s="26" t="str">
-        <f aca="false">IF(B27="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B27,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E27" s="26" t="str">
+      <c r="D27" s="27" t="str">
+        <f aca="false">IF(B27="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B27,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E27" s="27" t="str">
         <f aca="false">IF(B27="","",C27*D27)</f>
         <v/>
       </c>
-      <c r="F27" s="27" t="str">
-        <f aca="false">IF(B27="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B27,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G27" s="27" t="str">
-        <f aca="false">IF(B27="","",C27*INDEX(קטלוג!$G$5:$G$28,MATCH(B27,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F27" s="28" t="str">
+        <f aca="false">IF(B27="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B27,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G27" s="28" t="str">
+        <f aca="false">IF(B27="","",C27*INDEX(קטלוג!$G$5:$G$31,MATCH(B27,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3556,20 +3726,20 @@
       <c r="A28" s="13"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
-      <c r="D28" s="26" t="str">
-        <f aca="false">IF(B28="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B28,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E28" s="26" t="str">
+      <c r="D28" s="27" t="str">
+        <f aca="false">IF(B28="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B28,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E28" s="27" t="str">
         <f aca="false">IF(B28="","",C28*D28)</f>
         <v/>
       </c>
-      <c r="F28" s="27" t="str">
-        <f aca="false">IF(B28="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B28,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G28" s="27" t="str">
-        <f aca="false">IF(B28="","",C28*INDEX(קטלוג!$G$5:$G$28,MATCH(B28,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F28" s="28" t="str">
+        <f aca="false">IF(B28="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B28,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G28" s="28" t="str">
+        <f aca="false">IF(B28="","",C28*INDEX(קטלוג!$G$5:$G$31,MATCH(B28,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3577,20 +3747,20 @@
       <c r="A29" s="13"/>
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
-      <c r="D29" s="26" t="str">
-        <f aca="false">IF(B29="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B29,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E29" s="26" t="str">
+      <c r="D29" s="27" t="str">
+        <f aca="false">IF(B29="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B29,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E29" s="27" t="str">
         <f aca="false">IF(B29="","",C29*D29)</f>
         <v/>
       </c>
-      <c r="F29" s="27" t="str">
-        <f aca="false">IF(B29="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B29,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G29" s="27" t="str">
-        <f aca="false">IF(B29="","",C29*INDEX(קטלוג!$G$5:$G$28,MATCH(B29,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F29" s="28" t="str">
+        <f aca="false">IF(B29="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B29,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G29" s="28" t="str">
+        <f aca="false">IF(B29="","",C29*INDEX(קטלוג!$G$5:$G$31,MATCH(B29,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3598,20 +3768,20 @@
       <c r="A30" s="13"/>
       <c r="B30" s="13"/>
       <c r="C30" s="13"/>
-      <c r="D30" s="26" t="str">
-        <f aca="false">IF(B30="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B30,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E30" s="26" t="str">
+      <c r="D30" s="27" t="str">
+        <f aca="false">IF(B30="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B30,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E30" s="27" t="str">
         <f aca="false">IF(B30="","",C30*D30)</f>
         <v/>
       </c>
-      <c r="F30" s="27" t="str">
-        <f aca="false">IF(B30="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B30,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G30" s="27" t="str">
-        <f aca="false">IF(B30="","",C30*INDEX(קטלוג!$G$5:$G$28,MATCH(B30,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F30" s="28" t="str">
+        <f aca="false">IF(B30="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B30,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G30" s="28" t="str">
+        <f aca="false">IF(B30="","",C30*INDEX(קטלוג!$G$5:$G$31,MATCH(B30,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3619,20 +3789,20 @@
       <c r="A31" s="13"/>
       <c r="B31" s="13"/>
       <c r="C31" s="13"/>
-      <c r="D31" s="26" t="str">
-        <f aca="false">IF(B31="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B31,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E31" s="26" t="str">
+      <c r="D31" s="27" t="str">
+        <f aca="false">IF(B31="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B31,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E31" s="27" t="str">
         <f aca="false">IF(B31="","",C31*D31)</f>
         <v/>
       </c>
-      <c r="F31" s="27" t="str">
-        <f aca="false">IF(B31="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B31,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G31" s="27" t="str">
-        <f aca="false">IF(B31="","",C31*INDEX(קטלוג!$G$5:$G$28,MATCH(B31,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F31" s="28" t="str">
+        <f aca="false">IF(B31="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B31,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G31" s="28" t="str">
+        <f aca="false">IF(B31="","",C31*INDEX(קטלוג!$G$5:$G$31,MATCH(B31,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3640,20 +3810,20 @@
       <c r="A32" s="13"/>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
-      <c r="D32" s="26" t="str">
-        <f aca="false">IF(B32="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B32,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E32" s="26" t="str">
+      <c r="D32" s="27" t="str">
+        <f aca="false">IF(B32="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B32,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E32" s="27" t="str">
         <f aca="false">IF(B32="","",C32*D32)</f>
         <v/>
       </c>
-      <c r="F32" s="27" t="str">
-        <f aca="false">IF(B32="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B32,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G32" s="27" t="str">
-        <f aca="false">IF(B32="","",C32*INDEX(קטלוג!$G$5:$G$28,MATCH(B32,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F32" s="28" t="str">
+        <f aca="false">IF(B32="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B32,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G32" s="28" t="str">
+        <f aca="false">IF(B32="","",C32*INDEX(קטלוג!$G$5:$G$31,MATCH(B32,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3661,20 +3831,20 @@
       <c r="A33" s="13"/>
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
-      <c r="D33" s="26" t="str">
-        <f aca="false">IF(B33="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B33,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E33" s="26" t="str">
+      <c r="D33" s="27" t="str">
+        <f aca="false">IF(B33="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B33,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E33" s="27" t="str">
         <f aca="false">IF(B33="","",C33*D33)</f>
         <v/>
       </c>
-      <c r="F33" s="27" t="str">
-        <f aca="false">IF(B33="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B33,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G33" s="27" t="str">
-        <f aca="false">IF(B33="","",C33*INDEX(קטלוג!$G$5:$G$28,MATCH(B33,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F33" s="28" t="str">
+        <f aca="false">IF(B33="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B33,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G33" s="28" t="str">
+        <f aca="false">IF(B33="","",C33*INDEX(קטלוג!$G$5:$G$31,MATCH(B33,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3682,20 +3852,20 @@
       <c r="A34" s="13"/>
       <c r="B34" s="13"/>
       <c r="C34" s="13"/>
-      <c r="D34" s="26" t="str">
-        <f aca="false">IF(B34="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B34,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E34" s="26" t="str">
+      <c r="D34" s="27" t="str">
+        <f aca="false">IF(B34="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B34,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E34" s="27" t="str">
         <f aca="false">IF(B34="","",C34*D34)</f>
         <v/>
       </c>
-      <c r="F34" s="27" t="str">
-        <f aca="false">IF(B34="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B34,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G34" s="27" t="str">
-        <f aca="false">IF(B34="","",C34*INDEX(קטלוג!$G$5:$G$28,MATCH(B34,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F34" s="28" t="str">
+        <f aca="false">IF(B34="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B34,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G34" s="28" t="str">
+        <f aca="false">IF(B34="","",C34*INDEX(קטלוג!$G$5:$G$31,MATCH(B34,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3703,20 +3873,20 @@
       <c r="A35" s="13"/>
       <c r="B35" s="13"/>
       <c r="C35" s="13"/>
-      <c r="D35" s="26" t="str">
-        <f aca="false">IF(B35="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B35,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E35" s="26" t="str">
+      <c r="D35" s="27" t="str">
+        <f aca="false">IF(B35="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B35,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E35" s="27" t="str">
         <f aca="false">IF(B35="","",C35*D35)</f>
         <v/>
       </c>
-      <c r="F35" s="27" t="str">
-        <f aca="false">IF(B35="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B35,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G35" s="27" t="str">
-        <f aca="false">IF(B35="","",C35*INDEX(קטלוג!$G$5:$G$28,MATCH(B35,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F35" s="28" t="str">
+        <f aca="false">IF(B35="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B35,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G35" s="28" t="str">
+        <f aca="false">IF(B35="","",C35*INDEX(קטלוג!$G$5:$G$31,MATCH(B35,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3724,20 +3894,20 @@
       <c r="A36" s="13"/>
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
-      <c r="D36" s="26" t="str">
-        <f aca="false">IF(B36="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B36,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E36" s="26" t="str">
+      <c r="D36" s="27" t="str">
+        <f aca="false">IF(B36="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B36,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E36" s="27" t="str">
         <f aca="false">IF(B36="","",C36*D36)</f>
         <v/>
       </c>
-      <c r="F36" s="27" t="str">
-        <f aca="false">IF(B36="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B36,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G36" s="27" t="str">
-        <f aca="false">IF(B36="","",C36*INDEX(קטלוג!$G$5:$G$28,MATCH(B36,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F36" s="28" t="str">
+        <f aca="false">IF(B36="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B36,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G36" s="28" t="str">
+        <f aca="false">IF(B36="","",C36*INDEX(קטלוג!$G$5:$G$31,MATCH(B36,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3745,20 +3915,20 @@
       <c r="A37" s="13"/>
       <c r="B37" s="13"/>
       <c r="C37" s="13"/>
-      <c r="D37" s="26" t="str">
-        <f aca="false">IF(B37="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B37,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E37" s="26" t="str">
+      <c r="D37" s="27" t="str">
+        <f aca="false">IF(B37="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B37,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E37" s="27" t="str">
         <f aca="false">IF(B37="","",C37*D37)</f>
         <v/>
       </c>
-      <c r="F37" s="27" t="str">
-        <f aca="false">IF(B37="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B37,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G37" s="27" t="str">
-        <f aca="false">IF(B37="","",C37*INDEX(קטלוג!$G$5:$G$28,MATCH(B37,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F37" s="28" t="str">
+        <f aca="false">IF(B37="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B37,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G37" s="28" t="str">
+        <f aca="false">IF(B37="","",C37*INDEX(קטלוג!$G$5:$G$31,MATCH(B37,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3766,20 +3936,20 @@
       <c r="A38" s="13"/>
       <c r="B38" s="13"/>
       <c r="C38" s="13"/>
-      <c r="D38" s="26" t="str">
-        <f aca="false">IF(B38="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B38,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E38" s="26" t="str">
+      <c r="D38" s="27" t="str">
+        <f aca="false">IF(B38="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B38,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E38" s="27" t="str">
         <f aca="false">IF(B38="","",C38*D38)</f>
         <v/>
       </c>
-      <c r="F38" s="27" t="str">
-        <f aca="false">IF(B38="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B38,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G38" s="27" t="str">
-        <f aca="false">IF(B38="","",C38*INDEX(קטלוג!$G$5:$G$28,MATCH(B38,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F38" s="28" t="str">
+        <f aca="false">IF(B38="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B38,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G38" s="28" t="str">
+        <f aca="false">IF(B38="","",C38*INDEX(קטלוג!$G$5:$G$31,MATCH(B38,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3787,20 +3957,20 @@
       <c r="A39" s="13"/>
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
-      <c r="D39" s="26" t="str">
-        <f aca="false">IF(B39="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B39,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E39" s="26" t="str">
+      <c r="D39" s="27" t="str">
+        <f aca="false">IF(B39="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B39,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E39" s="27" t="str">
         <f aca="false">IF(B39="","",C39*D39)</f>
         <v/>
       </c>
-      <c r="F39" s="27" t="str">
-        <f aca="false">IF(B39="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B39,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G39" s="27" t="str">
-        <f aca="false">IF(B39="","",C39*INDEX(קטלוג!$G$5:$G$28,MATCH(B39,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F39" s="28" t="str">
+        <f aca="false">IF(B39="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B39,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G39" s="28" t="str">
+        <f aca="false">IF(B39="","",C39*INDEX(קטלוג!$G$5:$G$31,MATCH(B39,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3808,20 +3978,20 @@
       <c r="A40" s="13"/>
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
-      <c r="D40" s="26" t="str">
-        <f aca="false">IF(B40="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B40,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E40" s="26" t="str">
+      <c r="D40" s="27" t="str">
+        <f aca="false">IF(B40="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B40,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E40" s="27" t="str">
         <f aca="false">IF(B40="","",C40*D40)</f>
         <v/>
       </c>
-      <c r="F40" s="27" t="str">
-        <f aca="false">IF(B40="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B40,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G40" s="27" t="str">
-        <f aca="false">IF(B40="","",C40*INDEX(קטלוג!$G$5:$G$28,MATCH(B40,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F40" s="28" t="str">
+        <f aca="false">IF(B40="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B40,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G40" s="28" t="str">
+        <f aca="false">IF(B40="","",C40*INDEX(קטלוג!$G$5:$G$31,MATCH(B40,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3829,20 +3999,20 @@
       <c r="A41" s="13"/>
       <c r="B41" s="13"/>
       <c r="C41" s="13"/>
-      <c r="D41" s="26" t="str">
-        <f aca="false">IF(B41="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B41,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E41" s="26" t="str">
+      <c r="D41" s="27" t="str">
+        <f aca="false">IF(B41="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B41,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E41" s="27" t="str">
         <f aca="false">IF(B41="","",C41*D41)</f>
         <v/>
       </c>
-      <c r="F41" s="27" t="str">
-        <f aca="false">IF(B41="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B41,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G41" s="27" t="str">
-        <f aca="false">IF(B41="","",C41*INDEX(קטלוג!$G$5:$G$28,MATCH(B41,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F41" s="28" t="str">
+        <f aca="false">IF(B41="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B41,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G41" s="28" t="str">
+        <f aca="false">IF(B41="","",C41*INDEX(קטלוג!$G$5:$G$31,MATCH(B41,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3850,20 +4020,20 @@
       <c r="A42" s="13"/>
       <c r="B42" s="13"/>
       <c r="C42" s="13"/>
-      <c r="D42" s="26" t="str">
-        <f aca="false">IF(B42="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B42,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E42" s="26" t="str">
+      <c r="D42" s="27" t="str">
+        <f aca="false">IF(B42="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B42,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E42" s="27" t="str">
         <f aca="false">IF(B42="","",C42*D42)</f>
         <v/>
       </c>
-      <c r="F42" s="27" t="str">
-        <f aca="false">IF(B42="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B42,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G42" s="27" t="str">
-        <f aca="false">IF(B42="","",C42*INDEX(קטלוג!$G$5:$G$28,MATCH(B42,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F42" s="28" t="str">
+        <f aca="false">IF(B42="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B42,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G42" s="28" t="str">
+        <f aca="false">IF(B42="","",C42*INDEX(קטלוג!$G$5:$G$31,MATCH(B42,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3871,20 +4041,20 @@
       <c r="A43" s="13"/>
       <c r="B43" s="13"/>
       <c r="C43" s="13"/>
-      <c r="D43" s="26" t="str">
-        <f aca="false">IF(B43="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B43,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E43" s="26" t="str">
+      <c r="D43" s="27" t="str">
+        <f aca="false">IF(B43="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B43,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E43" s="27" t="str">
         <f aca="false">IF(B43="","",C43*D43)</f>
         <v/>
       </c>
-      <c r="F43" s="27" t="str">
-        <f aca="false">IF(B43="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B43,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G43" s="27" t="str">
-        <f aca="false">IF(B43="","",C43*INDEX(קטלוג!$G$5:$G$28,MATCH(B43,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F43" s="28" t="str">
+        <f aca="false">IF(B43="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B43,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G43" s="28" t="str">
+        <f aca="false">IF(B43="","",C43*INDEX(קטלוג!$G$5:$G$31,MATCH(B43,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3892,20 +4062,20 @@
       <c r="A44" s="13"/>
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
-      <c r="D44" s="26" t="str">
-        <f aca="false">IF(B44="","",INDEX(קטלוג!$H$5:$H$28,MATCH(B44,קטלוג!$C$5:$C$28,0)))</f>
-        <v/>
-      </c>
-      <c r="E44" s="26" t="str">
+      <c r="D44" s="27" t="str">
+        <f aca="false">IF(B44="","",INDEX(קטלוג!$H$5:$H$31,MATCH(B44,קטלוג!$C$5:$C$31,0)))</f>
+        <v/>
+      </c>
+      <c r="E44" s="27" t="str">
         <f aca="false">IF(B44="","",C44*D44)</f>
         <v/>
       </c>
-      <c r="F44" s="27" t="str">
-        <f aca="false">IF(B44="","",IF(INDEX(קטלוג!$F$5:$F$28,MATCH(B44,קטלוג!$C$5:$C$28,0))&gt;0,1,0))</f>
-        <v/>
-      </c>
-      <c r="G44" s="27" t="str">
-        <f aca="false">IF(B44="","",C44*INDEX(קטלוג!$G$5:$G$28,MATCH(B44,קטלוג!$C$5:$C$28,0)))</f>
+      <c r="F44" s="28" t="str">
+        <f aca="false">IF(B44="","",IF(INDEX(קטלוג!$F$5:$F$31,MATCH(B44,קטלוג!$C$5:$C$31,0))&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="G44" s="28" t="str">
+        <f aca="false">IF(B44="","",C44*INDEX(קטלוג!$G$5:$G$31,MATCH(B44,קטלוג!$C$5:$C$31,0)))</f>
         <v/>
       </c>
     </row>
@@ -3920,11 +4090,11 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="10" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="B46" s="18" t="n">
         <f aca="false">SUM(E5:E44)</f>
-        <v>990</v>
+        <v>840</v>
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
@@ -3934,11 +4104,11 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="B47" s="18" t="n">
         <f aca="false">'חבילה בסיסית'!$D$10</f>
-        <v>3170</v>
+        <v>3100</v>
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
@@ -3948,7 +4118,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="10" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="B48" s="18" t="n">
         <f aca="false">IF(SUMPRODUCT((F5:F44=1)*1)&gt;0,הנחות!$B$7,0)</f>
@@ -3962,11 +4132,11 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="10" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="B49" s="20" t="n">
         <f aca="false">SUM(B46:B48)</f>
-        <v>4655</v>
+        <v>4435</v>
       </c>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
@@ -3976,9 +4146,9 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="B50" s="28" t="n">
+        <v>129</v>
+      </c>
+      <c r="B50" s="29" t="n">
         <f aca="false">'חבילה בסיסית'!$E$10+SUM(G5:G44)</f>
         <v>6</v>
       </c>
@@ -3990,7 +4160,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="10" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B51" s="20" t="n">
         <f aca="false">INDEX(ריטיינר!$C$4:$C$6,MATCH(B50,ריטיינר!$A$4:$A$6,1))</f>
@@ -4004,7 +4174,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>146</v>
+        <v>161</v>
       </c>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
@@ -4016,7 +4186,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
-      <formula1>קטלוג!$C$5:$C$28</formula1>
+      <formula1>קטלוג!$C$5:$C$31</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>